<commit_message>
feat(v7.4.9): NWM Foerderzeitraeume, KPT NWM-Integration, Arbeitsplan Jahresnavigation
</commit_message>
<xml_diff>
--- a/Vorlagen/FuE-Stundenerfassung FZul VORLAGE NEU.xlsx
+++ b/Vorlagen/FuE-Stundenerfassung FZul VORLAGE NEU.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11130"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10404"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://cubinteccom-my.sharepoint.com/personal/m_ditscherlein_cubintec_com/Documents/Dokumente/Projekte/FZul/Stundenerfassung/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/mdbs/Documents/Dev/pze/Vorlagen/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="2" documentId="8_{E77D79BA-90C6-BA40-A097-BE79DA2CBB3D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{7CCBDB7B-89DD-EF45-A79A-8AA2FEC2F902}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7419E94B-931F-FF47-A60F-037F6DB3830F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-35300" yWindow="-28180" windowWidth="46320" windowHeight="28180" xr2:uid="{4E0623F2-5C98-4C26-BE2A-0325B7E83702}"/>
+    <workbookView xWindow="17720" yWindow="-21000" windowWidth="33480" windowHeight="21000" xr2:uid="{4E0623F2-5C98-4C26-BE2A-0325B7E83702}"/>
   </bookViews>
   <sheets>
     <sheet name="MA1" sheetId="1" r:id="rId1"/>
@@ -1679,34 +1679,277 @@
     <xf numFmtId="165" fontId="0" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="29" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="2" fontId="1" fillId="2" borderId="36" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="1" fillId="2" borderId="37" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="1" fillId="2" borderId="40" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="36" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="37" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="38" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="41" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="37" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="40" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="9" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="10" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="7" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="6" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="8" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="0" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="0" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="0" fillId="5" borderId="11" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="1" fontId="0" fillId="5" borderId="2" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="1" fontId="0" fillId="5" borderId="12" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="1" fontId="0" fillId="5" borderId="9" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="1" fontId="0" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="1" fontId="0" fillId="5" borderId="10" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="45" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="31" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="12" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="28" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="29" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="30" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="46" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" textRotation="90"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="49" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="50" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="11" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="32" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="2" borderId="41" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="2" borderId="37" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="2" borderId="40" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="167" fontId="7" fillId="5" borderId="36" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="167" fontId="7" fillId="5" borderId="37" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="167" fontId="7" fillId="5" borderId="40" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="1" fontId="0" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="0" fillId="0" borderId="12" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="35" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="1" fillId="3" borderId="36" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="1" fillId="3" borderId="37" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="1" fillId="3" borderId="38" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="32" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="36" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="37" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="38" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="0" fillId="2" borderId="36" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="0" fillId="2" borderId="37" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="0" fillId="2" borderId="40" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="39" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="1" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="1" fillId="0" borderId="26" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="25" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="13" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="164" fontId="0" fillId="2" borderId="20" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1716,12 +1959,6 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="166" fontId="13" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="1" fontId="9" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
@@ -1735,9 +1972,6 @@
       <alignment horizontal="center" vertical="center"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -1757,272 +1991,38 @@
       <alignment horizontal="left" vertical="center"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="2" fontId="1" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="29" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="2" fontId="1" fillId="0" borderId="26" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="25" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="39" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="11" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="45" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="32" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="46" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" textRotation="90"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="49" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="50" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="9" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="10" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="1" fontId="0" fillId="5" borderId="9" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="1" fontId="0" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="1" fontId="0" fillId="5" borderId="10" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="32" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="36" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="37" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="38" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="3" fontId="0" fillId="2" borderId="36" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="3" fontId="0" fillId="2" borderId="37" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="3" fontId="0" fillId="2" borderId="40" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="31" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="12" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="28" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="29" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="30" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="2" borderId="41" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="2" borderId="37" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="2" borderId="40" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="167" fontId="7" fillId="5" borderId="36" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="167" fontId="7" fillId="5" borderId="37" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="167" fontId="7" fillId="5" borderId="40" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="1" fontId="0" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="1" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="1" fontId="0" fillId="0" borderId="12" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="35" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="1" fillId="3" borderId="36" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="1" fillId="3" borderId="37" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="1" fillId="3" borderId="38" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="7" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="6" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="8" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="1" fillId="2" borderId="36" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="1" fillId="2" borderId="37" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="1" fillId="2" borderId="40" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="36" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="37" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="38" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="41" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="37" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="40" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="1" fontId="0" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="1" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="1" fontId="0" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="1" fontId="0" fillId="5" borderId="11" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="1" fontId="0" fillId="5" borderId="2" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="1" fontId="0" fillId="5" borderId="12" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -2792,42 +2792,42 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:52" s="2" customFormat="1" ht="16.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A1" s="110" t="s">
+      <c r="A1" s="160" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="110"/>
-      <c r="C1" s="110"/>
-      <c r="D1" s="110"/>
-      <c r="E1" s="110"/>
-      <c r="F1" s="110"/>
-      <c r="G1" s="110"/>
-      <c r="H1" s="110"/>
-      <c r="I1" s="110"/>
-      <c r="J1" s="110"/>
-      <c r="K1" s="110"/>
-      <c r="L1" s="110"/>
-      <c r="M1" s="110"/>
-      <c r="N1" s="110"/>
-      <c r="O1" s="110"/>
-      <c r="P1" s="110"/>
-      <c r="Q1" s="110"/>
-      <c r="R1" s="110"/>
-      <c r="S1" s="110"/>
-      <c r="T1" s="110"/>
-      <c r="U1" s="110"/>
-      <c r="V1" s="110"/>
-      <c r="W1" s="110"/>
-      <c r="X1" s="110"/>
-      <c r="Y1" s="110"/>
-      <c r="Z1" s="110"/>
-      <c r="AA1" s="110"/>
-      <c r="AB1" s="110"/>
-      <c r="AC1" s="110"/>
-      <c r="AD1" s="110"/>
-      <c r="AE1" s="110"/>
-      <c r="AF1" s="110"/>
-      <c r="AG1" s="110"/>
-      <c r="AH1" s="110"/>
+      <c r="B1" s="160"/>
+      <c r="C1" s="160"/>
+      <c r="D1" s="160"/>
+      <c r="E1" s="160"/>
+      <c r="F1" s="160"/>
+      <c r="G1" s="160"/>
+      <c r="H1" s="160"/>
+      <c r="I1" s="160"/>
+      <c r="J1" s="160"/>
+      <c r="K1" s="160"/>
+      <c r="L1" s="160"/>
+      <c r="M1" s="160"/>
+      <c r="N1" s="160"/>
+      <c r="O1" s="160"/>
+      <c r="P1" s="160"/>
+      <c r="Q1" s="160"/>
+      <c r="R1" s="160"/>
+      <c r="S1" s="160"/>
+      <c r="T1" s="160"/>
+      <c r="U1" s="160"/>
+      <c r="V1" s="160"/>
+      <c r="W1" s="160"/>
+      <c r="X1" s="160"/>
+      <c r="Y1" s="160"/>
+      <c r="Z1" s="160"/>
+      <c r="AA1" s="160"/>
+      <c r="AB1" s="160"/>
+      <c r="AC1" s="160"/>
+      <c r="AD1" s="160"/>
+      <c r="AE1" s="160"/>
+      <c r="AF1" s="160"/>
+      <c r="AG1" s="160"/>
+      <c r="AH1" s="160"/>
       <c r="AI1" s="18"/>
       <c r="AJ1" s="18"/>
       <c r="AK1" s="62"/>
@@ -2840,40 +2840,40 @@
       <c r="AW1" s="37"/>
     </row>
     <row r="2" spans="1:52" s="2" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A2" s="110"/>
-      <c r="B2" s="110"/>
-      <c r="C2" s="110"/>
-      <c r="D2" s="110"/>
-      <c r="E2" s="110"/>
-      <c r="F2" s="110"/>
-      <c r="G2" s="110"/>
-      <c r="H2" s="110"/>
-      <c r="I2" s="110"/>
-      <c r="J2" s="110"/>
-      <c r="K2" s="110"/>
-      <c r="L2" s="110"/>
-      <c r="M2" s="110"/>
-      <c r="N2" s="110"/>
-      <c r="O2" s="110"/>
-      <c r="P2" s="110"/>
-      <c r="Q2" s="110"/>
-      <c r="R2" s="110"/>
-      <c r="S2" s="110"/>
-      <c r="T2" s="110"/>
-      <c r="U2" s="110"/>
-      <c r="V2" s="110"/>
-      <c r="W2" s="110"/>
-      <c r="X2" s="110"/>
-      <c r="Y2" s="110"/>
-      <c r="Z2" s="110"/>
-      <c r="AA2" s="110"/>
-      <c r="AB2" s="110"/>
-      <c r="AC2" s="110"/>
-      <c r="AD2" s="110"/>
-      <c r="AE2" s="110"/>
-      <c r="AF2" s="110"/>
-      <c r="AG2" s="110"/>
-      <c r="AH2" s="110"/>
+      <c r="A2" s="160"/>
+      <c r="B2" s="160"/>
+      <c r="C2" s="160"/>
+      <c r="D2" s="160"/>
+      <c r="E2" s="160"/>
+      <c r="F2" s="160"/>
+      <c r="G2" s="160"/>
+      <c r="H2" s="160"/>
+      <c r="I2" s="160"/>
+      <c r="J2" s="160"/>
+      <c r="K2" s="160"/>
+      <c r="L2" s="160"/>
+      <c r="M2" s="160"/>
+      <c r="N2" s="160"/>
+      <c r="O2" s="160"/>
+      <c r="P2" s="160"/>
+      <c r="Q2" s="160"/>
+      <c r="R2" s="160"/>
+      <c r="S2" s="160"/>
+      <c r="T2" s="160"/>
+      <c r="U2" s="160"/>
+      <c r="V2" s="160"/>
+      <c r="W2" s="160"/>
+      <c r="X2" s="160"/>
+      <c r="Y2" s="160"/>
+      <c r="Z2" s="160"/>
+      <c r="AA2" s="160"/>
+      <c r="AB2" s="160"/>
+      <c r="AC2" s="160"/>
+      <c r="AD2" s="160"/>
+      <c r="AE2" s="160"/>
+      <c r="AF2" s="160"/>
+      <c r="AG2" s="160"/>
+      <c r="AH2" s="160"/>
       <c r="AK2" s="37"/>
       <c r="AO2" s="37"/>
       <c r="AP2" s="37"/>
@@ -2883,47 +2883,47 @@
       <c r="AW2" s="37"/>
     </row>
     <row r="3" spans="1:52" s="2" customFormat="1" ht="25.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A3" s="95" t="s">
-        <v>1</v>
-      </c>
-      <c r="B3" s="95"/>
-      <c r="C3" s="95"/>
-      <c r="D3" s="95"/>
-      <c r="E3" s="95"/>
-      <c r="F3" s="95"/>
-      <c r="G3" s="95"/>
-      <c r="H3" s="95"/>
-      <c r="I3" s="111" t="s">
+      <c r="A3" s="170" t="s">
+        <v>1</v>
+      </c>
+      <c r="B3" s="170"/>
+      <c r="C3" s="170"/>
+      <c r="D3" s="170"/>
+      <c r="E3" s="170"/>
+      <c r="F3" s="170"/>
+      <c r="G3" s="170"/>
+      <c r="H3" s="170"/>
+      <c r="I3" s="161" t="s">
         <v>134</v>
       </c>
-      <c r="J3" s="111"/>
-      <c r="K3" s="111"/>
-      <c r="L3" s="111"/>
-      <c r="M3" s="111"/>
-      <c r="N3" s="111"/>
-      <c r="O3" s="111"/>
-      <c r="P3" s="111"/>
-      <c r="Q3" s="111"/>
-      <c r="R3" s="111"/>
-      <c r="S3" s="111"/>
-      <c r="T3" s="111"/>
-      <c r="U3" s="111"/>
-      <c r="V3" s="111"/>
-      <c r="W3" s="111"/>
-      <c r="X3" s="111"/>
-      <c r="Y3" s="97" t="s">
+      <c r="J3" s="161"/>
+      <c r="K3" s="161"/>
+      <c r="L3" s="161"/>
+      <c r="M3" s="161"/>
+      <c r="N3" s="161"/>
+      <c r="O3" s="161"/>
+      <c r="P3" s="161"/>
+      <c r="Q3" s="161"/>
+      <c r="R3" s="161"/>
+      <c r="S3" s="161"/>
+      <c r="T3" s="161"/>
+      <c r="U3" s="161"/>
+      <c r="V3" s="161"/>
+      <c r="W3" s="161"/>
+      <c r="X3" s="161"/>
+      <c r="Y3" s="163" t="s">
         <v>2</v>
       </c>
-      <c r="Z3" s="97"/>
-      <c r="AA3" s="97"/>
-      <c r="AB3" s="97"/>
-      <c r="AC3" s="97"/>
-      <c r="AD3" s="94">
+      <c r="Z3" s="163"/>
+      <c r="AA3" s="163"/>
+      <c r="AB3" s="163"/>
+      <c r="AC3" s="163"/>
+      <c r="AD3" s="169">
         <v>2020</v>
       </c>
-      <c r="AE3" s="94"/>
-      <c r="AF3" s="94"/>
-      <c r="AG3" s="94"/>
+      <c r="AE3" s="169"/>
+      <c r="AF3" s="169"/>
+      <c r="AG3" s="169"/>
       <c r="AH3" s="17">
         <f>IF((MOD(YEAR(A10),4)=0)-(MOD(YEAR(A10),100)=0)+(MOD(YEAR(A10),400)=0)=0,0,1)</f>
         <v>1</v>
@@ -2937,48 +2937,48 @@
       <c r="AW3" s="37"/>
     </row>
     <row r="4" spans="1:52" s="2" customFormat="1" ht="25.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A4" s="95" t="s">
+      <c r="A4" s="170" t="s">
         <v>3</v>
       </c>
-      <c r="B4" s="95"/>
-      <c r="C4" s="95"/>
-      <c r="D4" s="95"/>
-      <c r="E4" s="95"/>
-      <c r="F4" s="95"/>
-      <c r="G4" s="95"/>
-      <c r="H4" s="95"/>
-      <c r="I4" s="112" t="s">
+      <c r="B4" s="170"/>
+      <c r="C4" s="170"/>
+      <c r="D4" s="170"/>
+      <c r="E4" s="170"/>
+      <c r="F4" s="170"/>
+      <c r="G4" s="170"/>
+      <c r="H4" s="170"/>
+      <c r="I4" s="162" t="s">
         <v>135</v>
       </c>
-      <c r="J4" s="112"/>
-      <c r="K4" s="112"/>
-      <c r="L4" s="112"/>
-      <c r="M4" s="112"/>
-      <c r="N4" s="112"/>
-      <c r="O4" s="112"/>
-      <c r="P4" s="112"/>
-      <c r="Q4" s="112"/>
-      <c r="R4" s="112"/>
-      <c r="S4" s="112"/>
-      <c r="T4" s="112"/>
-      <c r="U4" s="112"/>
-      <c r="V4" s="112"/>
-      <c r="W4" s="112"/>
-      <c r="X4" s="112"/>
-      <c r="Y4" s="97" t="s">
+      <c r="J4" s="162"/>
+      <c r="K4" s="162"/>
+      <c r="L4" s="162"/>
+      <c r="M4" s="162"/>
+      <c r="N4" s="162"/>
+      <c r="O4" s="162"/>
+      <c r="P4" s="162"/>
+      <c r="Q4" s="162"/>
+      <c r="R4" s="162"/>
+      <c r="S4" s="162"/>
+      <c r="T4" s="162"/>
+      <c r="U4" s="162"/>
+      <c r="V4" s="162"/>
+      <c r="W4" s="162"/>
+      <c r="X4" s="162"/>
+      <c r="Y4" s="163" t="s">
         <v>4</v>
       </c>
-      <c r="Z4" s="97"/>
-      <c r="AA4" s="97"/>
-      <c r="AB4" s="97"/>
-      <c r="AC4" s="97"/>
-      <c r="AD4" s="103" t="s">
+      <c r="Z4" s="163"/>
+      <c r="AA4" s="163"/>
+      <c r="AB4" s="163"/>
+      <c r="AC4" s="163"/>
+      <c r="AD4" s="177" t="s">
         <v>20</v>
       </c>
-      <c r="AE4" s="103"/>
-      <c r="AF4" s="103"/>
-      <c r="AG4" s="103"/>
-      <c r="AH4" s="103"/>
+      <c r="AE4" s="177"/>
+      <c r="AF4" s="177"/>
+      <c r="AG4" s="177"/>
+      <c r="AH4" s="177"/>
       <c r="AK4" s="37"/>
       <c r="AO4" s="37"/>
       <c r="AP4" s="37"/>
@@ -2988,42 +2988,42 @@
       <c r="AW4" s="37"/>
     </row>
     <row r="5" spans="1:52" s="2" customFormat="1" ht="25.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A5" s="113" t="s">
+      <c r="A5" s="164" t="s">
         <v>6</v>
       </c>
-      <c r="B5" s="113"/>
-      <c r="C5" s="113"/>
-      <c r="D5" s="113"/>
-      <c r="E5" s="113"/>
-      <c r="F5" s="113"/>
-      <c r="G5" s="113"/>
-      <c r="H5" s="113"/>
-      <c r="I5" s="113"/>
-      <c r="J5" s="113"/>
-      <c r="K5" s="113"/>
-      <c r="L5" s="113"/>
-      <c r="M5" s="113"/>
-      <c r="N5" s="113"/>
-      <c r="O5" s="113"/>
-      <c r="P5" s="113"/>
-      <c r="Q5" s="113"/>
-      <c r="R5" s="113"/>
-      <c r="S5" s="113"/>
-      <c r="T5" s="113"/>
-      <c r="U5" s="113"/>
-      <c r="V5" s="113"/>
-      <c r="W5" s="113"/>
-      <c r="X5" s="113"/>
-      <c r="Y5" s="113"/>
-      <c r="Z5" s="113"/>
-      <c r="AA5" s="113"/>
-      <c r="AB5" s="113"/>
-      <c r="AC5" s="113"/>
-      <c r="AD5" s="113"/>
-      <c r="AE5" s="113"/>
-      <c r="AF5" s="113"/>
-      <c r="AG5" s="113"/>
-      <c r="AH5" s="113"/>
+      <c r="B5" s="164"/>
+      <c r="C5" s="164"/>
+      <c r="D5" s="164"/>
+      <c r="E5" s="164"/>
+      <c r="F5" s="164"/>
+      <c r="G5" s="164"/>
+      <c r="H5" s="164"/>
+      <c r="I5" s="164"/>
+      <c r="J5" s="164"/>
+      <c r="K5" s="164"/>
+      <c r="L5" s="164"/>
+      <c r="M5" s="164"/>
+      <c r="N5" s="164"/>
+      <c r="O5" s="164"/>
+      <c r="P5" s="164"/>
+      <c r="Q5" s="164"/>
+      <c r="R5" s="164"/>
+      <c r="S5" s="164"/>
+      <c r="T5" s="164"/>
+      <c r="U5" s="164"/>
+      <c r="V5" s="164"/>
+      <c r="W5" s="164"/>
+      <c r="X5" s="164"/>
+      <c r="Y5" s="164"/>
+      <c r="Z5" s="164"/>
+      <c r="AA5" s="164"/>
+      <c r="AB5" s="164"/>
+      <c r="AC5" s="164"/>
+      <c r="AD5" s="164"/>
+      <c r="AE5" s="164"/>
+      <c r="AF5" s="164"/>
+      <c r="AG5" s="164"/>
+      <c r="AH5" s="164"/>
       <c r="AK5" s="37"/>
       <c r="AO5" s="37"/>
       <c r="AP5" s="37"/>
@@ -3037,49 +3037,49 @@
       <c r="A6" s="36" t="s">
         <v>7</v>
       </c>
-      <c r="B6" s="96" t="s">
+      <c r="B6" s="171" t="s">
         <v>131</v>
       </c>
-      <c r="C6" s="96"/>
-      <c r="D6" s="96"/>
-      <c r="E6" s="96"/>
-      <c r="F6" s="96"/>
-      <c r="G6" s="96"/>
-      <c r="H6" s="96"/>
-      <c r="I6" s="96"/>
-      <c r="J6" s="97" t="s">
+      <c r="C6" s="171"/>
+      <c r="D6" s="171"/>
+      <c r="E6" s="171"/>
+      <c r="F6" s="171"/>
+      <c r="G6" s="171"/>
+      <c r="H6" s="171"/>
+      <c r="I6" s="171"/>
+      <c r="J6" s="163" t="s">
         <v>8</v>
       </c>
-      <c r="K6" s="97"/>
-      <c r="L6" s="97"/>
-      <c r="M6" s="96" t="s">
+      <c r="K6" s="163"/>
+      <c r="L6" s="163"/>
+      <c r="M6" s="171" t="s">
         <v>132</v>
       </c>
-      <c r="N6" s="96"/>
-      <c r="O6" s="96"/>
-      <c r="P6" s="96"/>
-      <c r="Q6" s="96"/>
-      <c r="R6" s="96"/>
-      <c r="S6" s="96"/>
-      <c r="T6" s="96"/>
-      <c r="U6" s="97" t="s">
+      <c r="N6" s="171"/>
+      <c r="O6" s="171"/>
+      <c r="P6" s="171"/>
+      <c r="Q6" s="171"/>
+      <c r="R6" s="171"/>
+      <c r="S6" s="171"/>
+      <c r="T6" s="171"/>
+      <c r="U6" s="163" t="s">
         <v>9</v>
       </c>
-      <c r="V6" s="97"/>
-      <c r="W6" s="97"/>
-      <c r="X6" s="97"/>
-      <c r="Y6" s="97"/>
-      <c r="Z6" s="97"/>
-      <c r="AA6" s="97"/>
-      <c r="AB6" s="97"/>
-      <c r="AC6" s="97"/>
-      <c r="AD6" s="96" t="s">
+      <c r="V6" s="163"/>
+      <c r="W6" s="163"/>
+      <c r="X6" s="163"/>
+      <c r="Y6" s="163"/>
+      <c r="Z6" s="163"/>
+      <c r="AA6" s="163"/>
+      <c r="AB6" s="163"/>
+      <c r="AC6" s="163"/>
+      <c r="AD6" s="171" t="s">
         <v>133</v>
       </c>
-      <c r="AE6" s="96"/>
-      <c r="AF6" s="96"/>
-      <c r="AG6" s="96"/>
-      <c r="AH6" s="96"/>
+      <c r="AE6" s="171"/>
+      <c r="AF6" s="171"/>
+      <c r="AG6" s="171"/>
+      <c r="AH6" s="171"/>
       <c r="AK6" s="37"/>
       <c r="AO6" s="37"/>
       <c r="AP6" s="37"/>
@@ -3089,42 +3089,42 @@
       <c r="AW6" s="37"/>
     </row>
     <row r="7" spans="1:52" s="2" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A7" s="98" t="s">
+      <c r="A7" s="172" t="s">
         <v>10</v>
       </c>
-      <c r="B7" s="102" t="s">
+      <c r="B7" s="176" t="s">
         <v>11</v>
       </c>
-      <c r="C7" s="102"/>
-      <c r="D7" s="102"/>
-      <c r="E7" s="102"/>
-      <c r="F7" s="102"/>
-      <c r="G7" s="102"/>
-      <c r="H7" s="102"/>
-      <c r="I7" s="102"/>
-      <c r="J7" s="102"/>
-      <c r="K7" s="102"/>
-      <c r="L7" s="102"/>
-      <c r="M7" s="102"/>
-      <c r="N7" s="102"/>
-      <c r="O7" s="102"/>
-      <c r="P7" s="102"/>
-      <c r="Q7" s="102"/>
-      <c r="R7" s="102"/>
-      <c r="S7" s="102"/>
-      <c r="T7" s="102"/>
-      <c r="U7" s="102"/>
-      <c r="V7" s="102"/>
-      <c r="W7" s="102"/>
-      <c r="X7" s="102"/>
-      <c r="Y7" s="102"/>
-      <c r="Z7" s="102"/>
-      <c r="AA7" s="102"/>
-      <c r="AB7" s="102"/>
-      <c r="AC7" s="102"/>
-      <c r="AD7" s="102"/>
-      <c r="AE7" s="102"/>
-      <c r="AF7" s="102"/>
+      <c r="C7" s="176"/>
+      <c r="D7" s="176"/>
+      <c r="E7" s="176"/>
+      <c r="F7" s="176"/>
+      <c r="G7" s="176"/>
+      <c r="H7" s="176"/>
+      <c r="I7" s="176"/>
+      <c r="J7" s="176"/>
+      <c r="K7" s="176"/>
+      <c r="L7" s="176"/>
+      <c r="M7" s="176"/>
+      <c r="N7" s="176"/>
+      <c r="O7" s="176"/>
+      <c r="P7" s="176"/>
+      <c r="Q7" s="176"/>
+      <c r="R7" s="176"/>
+      <c r="S7" s="176"/>
+      <c r="T7" s="176"/>
+      <c r="U7" s="176"/>
+      <c r="V7" s="176"/>
+      <c r="W7" s="176"/>
+      <c r="X7" s="176"/>
+      <c r="Y7" s="176"/>
+      <c r="Z7" s="176"/>
+      <c r="AA7" s="176"/>
+      <c r="AB7" s="176"/>
+      <c r="AC7" s="176"/>
+      <c r="AD7" s="176"/>
+      <c r="AE7" s="176"/>
+      <c r="AF7" s="176"/>
       <c r="AG7" s="14"/>
       <c r="AH7" s="5"/>
       <c r="AI7"/>
@@ -3141,52 +3141,52 @@
       </c>
     </row>
     <row r="8" spans="1:52" x14ac:dyDescent="0.2">
-      <c r="A8" s="99"/>
-      <c r="B8" s="101" t="s">
+      <c r="A8" s="173"/>
+      <c r="B8" s="175" t="s">
         <v>12</v>
       </c>
-      <c r="C8" s="101"/>
-      <c r="D8" s="101"/>
-      <c r="E8" s="101"/>
-      <c r="F8" s="101"/>
-      <c r="G8" s="101"/>
-      <c r="H8" s="101"/>
-      <c r="I8" s="101"/>
-      <c r="J8" s="101"/>
-      <c r="K8" s="101"/>
-      <c r="L8" s="101"/>
-      <c r="M8" s="101"/>
-      <c r="N8" s="101"/>
-      <c r="O8" s="101"/>
-      <c r="P8" s="101"/>
-      <c r="Q8" s="101"/>
-      <c r="R8" s="101"/>
-      <c r="S8" s="101"/>
-      <c r="T8" s="101"/>
-      <c r="U8" s="101"/>
-      <c r="V8" s="101"/>
-      <c r="W8" s="101"/>
-      <c r="X8" s="101"/>
-      <c r="Y8" s="101"/>
-      <c r="Z8" s="101"/>
-      <c r="AA8" s="101"/>
-      <c r="AB8" s="101"/>
-      <c r="AC8" s="101"/>
-      <c r="AD8" s="101"/>
-      <c r="AE8" s="101"/>
-      <c r="AF8" s="101"/>
+      <c r="C8" s="175"/>
+      <c r="D8" s="175"/>
+      <c r="E8" s="175"/>
+      <c r="F8" s="175"/>
+      <c r="G8" s="175"/>
+      <c r="H8" s="175"/>
+      <c r="I8" s="175"/>
+      <c r="J8" s="175"/>
+      <c r="K8" s="175"/>
+      <c r="L8" s="175"/>
+      <c r="M8" s="175"/>
+      <c r="N8" s="175"/>
+      <c r="O8" s="175"/>
+      <c r="P8" s="175"/>
+      <c r="Q8" s="175"/>
+      <c r="R8" s="175"/>
+      <c r="S8" s="175"/>
+      <c r="T8" s="175"/>
+      <c r="U8" s="175"/>
+      <c r="V8" s="175"/>
+      <c r="W8" s="175"/>
+      <c r="X8" s="175"/>
+      <c r="Y8" s="175"/>
+      <c r="Z8" s="175"/>
+      <c r="AA8" s="175"/>
+      <c r="AB8" s="175"/>
+      <c r="AC8" s="175"/>
+      <c r="AD8" s="175"/>
+      <c r="AE8" s="175"/>
+      <c r="AF8" s="175"/>
       <c r="AG8" s="15"/>
       <c r="AH8" s="6"/>
-      <c r="AK8" s="86" t="s">
+      <c r="AK8" s="185" t="s">
         <v>13</v>
       </c>
-      <c r="AL8" s="86" t="s">
+      <c r="AL8" s="185" t="s">
         <v>14</v>
       </c>
       <c r="AM8" s="71"/>
     </row>
     <row r="9" spans="1:52" ht="16" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A9" s="100"/>
+      <c r="A9" s="174"/>
       <c r="B9" s="3">
         <v>1</v>
       </c>
@@ -3286,13 +3286,13 @@
       <c r="AH9" s="7" t="s">
         <v>16</v>
       </c>
-      <c r="AK9" s="86"/>
-      <c r="AL9" s="86"/>
+      <c r="AK9" s="185"/>
+      <c r="AL9" s="185"/>
       <c r="AM9" s="71"/>
       <c r="AT9" s="2"/>
     </row>
     <row r="10" spans="1:52" x14ac:dyDescent="0.2">
-      <c r="A10" s="89">
+      <c r="A10" s="166">
         <f>DATE($AD$3,1,1)</f>
         <v>43831</v>
       </c>
@@ -3420,7 +3420,7 @@
         <f t="shared" si="0"/>
         <v>6</v>
       </c>
-      <c r="AG10" s="92">
+      <c r="AG10" s="165">
         <f>SUM(B11:AF11)</f>
         <v>0</v>
       </c>
@@ -3442,10 +3442,10 @@
         <v>17</v>
       </c>
       <c r="AV10" s="59"/>
-      <c r="AW10" s="79" t="s">
+      <c r="AW10" s="178" t="s">
         <v>18</v>
       </c>
-      <c r="AX10" s="79"/>
+      <c r="AX10" s="178"/>
       <c r="AY10" s="60"/>
       <c r="AZ10" s="61">
         <f>$AD$3</f>
@@ -3453,7 +3453,7 @@
       </c>
     </row>
     <row r="11" spans="1:52" x14ac:dyDescent="0.2">
-      <c r="A11" s="89"/>
+      <c r="A11" s="166"/>
       <c r="B11" s="51"/>
       <c r="C11" s="50"/>
       <c r="D11" s="50"/>
@@ -3485,7 +3485,7 @@
       <c r="AD11" s="50"/>
       <c r="AE11" s="50"/>
       <c r="AF11" s="50"/>
-      <c r="AG11" s="92"/>
+      <c r="AG11" s="165"/>
       <c r="AH11" s="9" t="s">
         <v>19</v>
       </c>
@@ -3494,15 +3494,15 @@
         <v>20</v>
       </c>
       <c r="AV11" s="1"/>
-      <c r="AW11" s="93" t="s">
+      <c r="AW11" s="188" t="s">
         <v>21</v>
       </c>
-      <c r="AX11" s="93"/>
+      <c r="AX11" s="188"/>
       <c r="AY11" s="1"/>
       <c r="AZ11" s="44"/>
     </row>
     <row r="12" spans="1:52" x14ac:dyDescent="0.2">
-      <c r="A12" s="89">
+      <c r="A12" s="166">
         <f>EOMONTH(A10,0)+1</f>
         <v>43862</v>
       </c>
@@ -3622,9 +3622,9 @@
         <f t="shared" ref="AD12" si="2">WEEKDAY(DATE($AD$3,MONTH($A12),AD$9))</f>
         <v>7</v>
       </c>
-      <c r="AE12" s="91"/>
-      <c r="AF12" s="91"/>
-      <c r="AG12" s="92">
+      <c r="AE12" s="168"/>
+      <c r="AF12" s="168"/>
+      <c r="AG12" s="165">
         <f>SUM(B13:AF13)</f>
         <v>0</v>
       </c>
@@ -3673,7 +3673,7 @@
       </c>
     </row>
     <row r="13" spans="1:52" x14ac:dyDescent="0.2">
-      <c r="A13" s="90"/>
+      <c r="A13" s="167"/>
       <c r="B13" s="50"/>
       <c r="C13" s="50"/>
       <c r="D13" s="50"/>
@@ -3703,9 +3703,9 @@
       <c r="AB13" s="50"/>
       <c r="AC13" s="50"/>
       <c r="AD13" s="50"/>
-      <c r="AE13" s="91"/>
-      <c r="AF13" s="91"/>
-      <c r="AG13" s="92"/>
+      <c r="AE13" s="168"/>
+      <c r="AF13" s="168"/>
+      <c r="AG13" s="165"/>
       <c r="AH13" s="9" t="s">
         <v>19</v>
       </c>
@@ -3755,7 +3755,7 @@
       </c>
     </row>
     <row r="14" spans="1:52" x14ac:dyDescent="0.2">
-      <c r="A14" s="89">
+      <c r="A14" s="166">
         <f>EOMONTH(A12,0)+1</f>
         <v>43891</v>
       </c>
@@ -3883,7 +3883,7 @@
         <f t="shared" si="8"/>
         <v>3</v>
       </c>
-      <c r="AG14" s="92">
+      <c r="AG14" s="165">
         <f t="shared" ref="AG14" si="9">SUM(B15:AF15)</f>
         <v>0</v>
       </c>
@@ -3947,7 +3947,7 @@
       </c>
     </row>
     <row r="15" spans="1:52" x14ac:dyDescent="0.2">
-      <c r="A15" s="90"/>
+      <c r="A15" s="167"/>
       <c r="B15" s="50"/>
       <c r="C15" s="50"/>
       <c r="D15" s="50"/>
@@ -3979,7 +3979,7 @@
       <c r="AD15" s="50"/>
       <c r="AE15" s="50"/>
       <c r="AF15" s="50"/>
-      <c r="AG15" s="92"/>
+      <c r="AG15" s="165"/>
       <c r="AH15" s="9" t="s">
         <v>19</v>
       </c>
@@ -4030,7 +4030,7 @@
       </c>
     </row>
     <row r="16" spans="1:52" x14ac:dyDescent="0.2">
-      <c r="A16" s="89">
+      <c r="A16" s="166">
         <f t="shared" ref="A16" si="11">EOMONTH(A14,0)+1</f>
         <v>43922</v>
       </c>
@@ -4154,8 +4154,8 @@
         <f t="shared" si="12"/>
         <v>5</v>
       </c>
-      <c r="AF16" s="91"/>
-      <c r="AG16" s="92">
+      <c r="AF16" s="168"/>
+      <c r="AG16" s="165">
         <f t="shared" ref="AG16" si="13">SUM(B17:AF17)</f>
         <v>0</v>
       </c>
@@ -4220,7 +4220,7 @@
       </c>
     </row>
     <row r="17" spans="1:52" x14ac:dyDescent="0.2">
-      <c r="A17" s="90"/>
+      <c r="A17" s="167"/>
       <c r="B17" s="50"/>
       <c r="C17" s="50"/>
       <c r="D17" s="50"/>
@@ -4251,8 +4251,8 @@
       <c r="AC17" s="50"/>
       <c r="AD17" s="50"/>
       <c r="AE17" s="50"/>
-      <c r="AF17" s="91"/>
-      <c r="AG17" s="92"/>
+      <c r="AF17" s="168"/>
+      <c r="AG17" s="165"/>
       <c r="AH17" s="9" t="s">
         <v>19</v>
       </c>
@@ -4304,7 +4304,7 @@
       </c>
     </row>
     <row r="18" spans="1:52" x14ac:dyDescent="0.2">
-      <c r="A18" s="89">
+      <c r="A18" s="166">
         <f t="shared" ref="A18" si="14">EOMONTH(A16,0)+1</f>
         <v>43952</v>
       </c>
@@ -4432,7 +4432,7 @@
         <f t="shared" si="15"/>
         <v>PS</v>
       </c>
-      <c r="AG18" s="92">
+      <c r="AG18" s="165">
         <f t="shared" ref="AG18" si="16">SUM(B19:AF19)</f>
         <v>0</v>
       </c>
@@ -4497,7 +4497,7 @@
       </c>
     </row>
     <row r="19" spans="1:52" x14ac:dyDescent="0.2">
-      <c r="A19" s="90"/>
+      <c r="A19" s="167"/>
       <c r="B19" s="50"/>
       <c r="C19" s="50"/>
       <c r="D19" s="50"/>
@@ -4529,7 +4529,7 @@
       <c r="AD19" s="50"/>
       <c r="AE19" s="50"/>
       <c r="AF19" s="50"/>
-      <c r="AG19" s="92"/>
+      <c r="AG19" s="165"/>
       <c r="AH19" s="9" t="s">
         <v>19</v>
       </c>
@@ -4579,7 +4579,7 @@
       </c>
     </row>
     <row r="20" spans="1:52" x14ac:dyDescent="0.2">
-      <c r="A20" s="89">
+      <c r="A20" s="166">
         <f t="shared" ref="A20" si="18">EOMONTH(A18,0)+1</f>
         <v>43983</v>
       </c>
@@ -4703,8 +4703,8 @@
         <f t="shared" si="19"/>
         <v>3</v>
       </c>
-      <c r="AF20" s="91"/>
-      <c r="AG20" s="92">
+      <c r="AF20" s="168"/>
+      <c r="AG20" s="165">
         <f t="shared" ref="AG20" si="20">SUM(B21:AF21)</f>
         <v>0</v>
       </c>
@@ -4770,7 +4770,7 @@
       </c>
     </row>
     <row r="21" spans="1:52" x14ac:dyDescent="0.2">
-      <c r="A21" s="90"/>
+      <c r="A21" s="167"/>
       <c r="B21" s="50"/>
       <c r="C21" s="50"/>
       <c r="D21" s="50"/>
@@ -4801,8 +4801,8 @@
       <c r="AC21" s="50"/>
       <c r="AD21" s="50"/>
       <c r="AE21" s="50"/>
-      <c r="AF21" s="91"/>
-      <c r="AG21" s="92"/>
+      <c r="AF21" s="168"/>
+      <c r="AG21" s="165"/>
       <c r="AH21" s="9" t="s">
         <v>19</v>
       </c>
@@ -4854,7 +4854,7 @@
       </c>
     </row>
     <row r="22" spans="1:52" x14ac:dyDescent="0.2">
-      <c r="A22" s="89">
+      <c r="A22" s="166">
         <f t="shared" ref="A22" si="21">EOMONTH(A20,0)+1</f>
         <v>44013</v>
       </c>
@@ -4982,7 +4982,7 @@
         <f t="shared" si="22"/>
         <v>6</v>
       </c>
-      <c r="AG22" s="92">
+      <c r="AG22" s="165">
         <f t="shared" ref="AG22" si="23">SUM(B23:AF23)</f>
         <v>0</v>
       </c>
@@ -5047,7 +5047,7 @@
       </c>
     </row>
     <row r="23" spans="1:52" x14ac:dyDescent="0.2">
-      <c r="A23" s="90"/>
+      <c r="A23" s="167"/>
       <c r="B23" s="50"/>
       <c r="C23" s="50"/>
       <c r="D23" s="50"/>
@@ -5079,7 +5079,7 @@
       <c r="AD23" s="50"/>
       <c r="AE23" s="50"/>
       <c r="AF23" s="50"/>
-      <c r="AG23" s="92"/>
+      <c r="AG23" s="165"/>
       <c r="AH23" s="9" t="s">
         <v>19</v>
       </c>
@@ -5132,7 +5132,7 @@
       </c>
     </row>
     <row r="24" spans="1:52" x14ac:dyDescent="0.2">
-      <c r="A24" s="89">
+      <c r="A24" s="166">
         <f t="shared" ref="A24" si="24">EOMONTH(A22,0)+1</f>
         <v>44044</v>
       </c>
@@ -5260,7 +5260,7 @@
         <f t="shared" si="25"/>
         <v>2</v>
       </c>
-      <c r="AG24" s="92">
+      <c r="AG24" s="165">
         <f t="shared" ref="AG24" si="26">SUM(B25:AF25)</f>
         <v>65</v>
       </c>
@@ -5324,7 +5324,7 @@
       </c>
     </row>
     <row r="25" spans="1:52" x14ac:dyDescent="0.2">
-      <c r="A25" s="90"/>
+      <c r="A25" s="167"/>
       <c r="B25" s="50"/>
       <c r="C25" s="50"/>
       <c r="D25" s="50"/>
@@ -5386,7 +5386,7 @@
       <c r="AF25" s="50">
         <v>3</v>
       </c>
-      <c r="AG25" s="92"/>
+      <c r="AG25" s="165"/>
       <c r="AH25" s="9" t="s">
         <v>19</v>
       </c>
@@ -5436,7 +5436,7 @@
       </c>
     </row>
     <row r="26" spans="1:52" x14ac:dyDescent="0.2">
-      <c r="A26" s="89">
+      <c r="A26" s="166">
         <f t="shared" ref="A26" si="29">EOMONTH(A24,0)+1</f>
         <v>44075</v>
       </c>
@@ -5560,8 +5560,8 @@
         <f t="shared" si="30"/>
         <v>4</v>
       </c>
-      <c r="AF26" s="91"/>
-      <c r="AG26" s="92">
+      <c r="AF26" s="168"/>
+      <c r="AG26" s="165">
         <f t="shared" ref="AG26" si="31">SUM(B27:AF27)</f>
         <v>67</v>
       </c>
@@ -5625,7 +5625,7 @@
       </c>
     </row>
     <row r="27" spans="1:52" x14ac:dyDescent="0.2">
-      <c r="A27" s="90"/>
+      <c r="A27" s="167"/>
       <c r="B27" s="50">
         <v>4</v>
       </c>
@@ -5690,8 +5690,8 @@
       <c r="AE27" s="50">
         <v>2</v>
       </c>
-      <c r="AF27" s="91"/>
-      <c r="AG27" s="92"/>
+      <c r="AF27" s="168"/>
+      <c r="AG27" s="165"/>
       <c r="AH27" s="9" t="s">
         <v>19</v>
       </c>
@@ -5742,7 +5742,7 @@
       </c>
     </row>
     <row r="28" spans="1:52" x14ac:dyDescent="0.2">
-      <c r="A28" s="89">
+      <c r="A28" s="166">
         <f t="shared" ref="A28" si="33">EOMONTH(A26,0)+1</f>
         <v>44105</v>
       </c>
@@ -5870,7 +5870,7 @@
         <f t="shared" si="34"/>
         <v>7</v>
       </c>
-      <c r="AG28" s="92">
+      <c r="AG28" s="165">
         <f t="shared" ref="AG28" si="35">SUM(B29:AF29)</f>
         <v>59</v>
       </c>
@@ -5933,7 +5933,7 @@
       </c>
     </row>
     <row r="29" spans="1:52" x14ac:dyDescent="0.2">
-      <c r="A29" s="90"/>
+      <c r="A29" s="167"/>
       <c r="B29" s="50">
         <v>2</v>
       </c>
@@ -6001,7 +6001,7 @@
         <v>1</v>
       </c>
       <c r="AF29" s="50"/>
-      <c r="AG29" s="92"/>
+      <c r="AG29" s="165"/>
       <c r="AH29" s="9" t="s">
         <v>19</v>
       </c>
@@ -6051,7 +6051,7 @@
       </c>
     </row>
     <row r="30" spans="1:52" x14ac:dyDescent="0.2">
-      <c r="A30" s="89">
+      <c r="A30" s="166">
         <f t="shared" ref="A30:A32" si="36">EOMONTH(A28,0)+1</f>
         <v>44136</v>
       </c>
@@ -6175,8 +6175,8 @@
         <f t="shared" si="37"/>
         <v>2</v>
       </c>
-      <c r="AF30" s="91"/>
-      <c r="AG30" s="92">
+      <c r="AF30" s="168"/>
+      <c r="AG30" s="165">
         <f t="shared" ref="AG30" si="38">SUM(B31:AF31)</f>
         <v>54</v>
       </c>
@@ -6198,20 +6198,20 @@
       <c r="AR30" s="54"/>
       <c r="AS30" s="38"/>
       <c r="AT30" s="37"/>
-      <c r="AU30" s="80" t="s">
+      <c r="AU30" s="179" t="s">
         <v>55</v>
       </c>
-      <c r="AV30" s="81"/>
-      <c r="AW30" s="81"/>
-      <c r="AX30" s="81"/>
-      <c r="AY30" s="82"/>
-      <c r="AZ30" s="87">
+      <c r="AV30" s="180"/>
+      <c r="AW30" s="180"/>
+      <c r="AX30" s="180"/>
+      <c r="AY30" s="181"/>
+      <c r="AZ30" s="186">
         <f>SUM(AZ13:AZ29)</f>
         <v>9</v>
       </c>
     </row>
     <row r="31" spans="1:52" ht="16" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A31" s="90"/>
+      <c r="A31" s="167"/>
       <c r="B31" s="50"/>
       <c r="C31" s="50">
         <v>6</v>
@@ -6274,8 +6274,8 @@
       <c r="AE31" s="50">
         <v>1</v>
       </c>
-      <c r="AF31" s="91"/>
-      <c r="AG31" s="92"/>
+      <c r="AF31" s="168"/>
+      <c r="AG31" s="165"/>
       <c r="AH31" s="9" t="s">
         <v>19</v>
       </c>
@@ -6286,15 +6286,15 @@
       <c r="AR31" s="41"/>
       <c r="AS31" s="41"/>
       <c r="AT31" s="37"/>
-      <c r="AU31" s="83"/>
-      <c r="AV31" s="84"/>
-      <c r="AW31" s="84"/>
-      <c r="AX31" s="84"/>
-      <c r="AY31" s="85"/>
-      <c r="AZ31" s="88"/>
+      <c r="AU31" s="182"/>
+      <c r="AV31" s="183"/>
+      <c r="AW31" s="183"/>
+      <c r="AX31" s="183"/>
+      <c r="AY31" s="184"/>
+      <c r="AZ31" s="187"/>
     </row>
     <row r="32" spans="1:52" x14ac:dyDescent="0.2">
-      <c r="A32" s="89">
+      <c r="A32" s="166">
         <f t="shared" si="36"/>
         <v>44166</v>
       </c>
@@ -6422,7 +6422,7 @@
         <f t="shared" si="39"/>
         <v>5</v>
       </c>
-      <c r="AG32" s="92">
+      <c r="AG32" s="165">
         <f t="shared" ref="AG32" si="40">SUM(B33:AF33)</f>
         <v>52</v>
       </c>
@@ -6443,7 +6443,7 @@
       <c r="AU32" s="2"/>
     </row>
     <row r="33" spans="1:54" x14ac:dyDescent="0.2">
-      <c r="A33" s="90"/>
+      <c r="A33" s="167"/>
       <c r="B33" s="50">
         <v>4</v>
       </c>
@@ -6501,7 +6501,7 @@
       <c r="AD33" s="50"/>
       <c r="AE33" s="50"/>
       <c r="AF33" s="50"/>
-      <c r="AG33" s="92"/>
+      <c r="AG33" s="165"/>
       <c r="AH33" s="9" t="s">
         <v>19</v>
       </c>
@@ -6523,27 +6523,27 @@
       <c r="L34" s="4"/>
       <c r="M34" s="4"/>
       <c r="N34" s="4"/>
-      <c r="O34" s="106" t="s">
+      <c r="O34" s="156" t="s">
         <v>56</v>
       </c>
-      <c r="P34" s="106"/>
-      <c r="Q34" s="106"/>
-      <c r="R34" s="106"/>
-      <c r="S34" s="106"/>
-      <c r="T34" s="106"/>
-      <c r="U34" s="106"/>
-      <c r="V34" s="106"/>
-      <c r="W34" s="106"/>
-      <c r="X34" s="106"/>
-      <c r="Y34" s="106"/>
-      <c r="Z34" s="106"/>
-      <c r="AA34" s="106"/>
-      <c r="AB34" s="106"/>
-      <c r="AC34" s="106"/>
-      <c r="AD34" s="106"/>
-      <c r="AE34" s="106"/>
-      <c r="AF34" s="107"/>
-      <c r="AG34" s="104">
+      <c r="P34" s="156"/>
+      <c r="Q34" s="156"/>
+      <c r="R34" s="156"/>
+      <c r="S34" s="156"/>
+      <c r="T34" s="156"/>
+      <c r="U34" s="156"/>
+      <c r="V34" s="156"/>
+      <c r="W34" s="156"/>
+      <c r="X34" s="156"/>
+      <c r="Y34" s="156"/>
+      <c r="Z34" s="156"/>
+      <c r="AA34" s="156"/>
+      <c r="AB34" s="156"/>
+      <c r="AC34" s="156"/>
+      <c r="AD34" s="156"/>
+      <c r="AE34" s="156"/>
+      <c r="AF34" s="157"/>
+      <c r="AG34" s="154">
         <f>SUM(AG10:AG33)</f>
         <v>297</v>
       </c>
@@ -6566,25 +6566,25 @@
       <c r="L35" s="12"/>
       <c r="M35" s="12"/>
       <c r="N35" s="12"/>
-      <c r="O35" s="108"/>
-      <c r="P35" s="108"/>
-      <c r="Q35" s="108"/>
-      <c r="R35" s="108"/>
-      <c r="S35" s="108"/>
-      <c r="T35" s="108"/>
-      <c r="U35" s="108"/>
-      <c r="V35" s="108"/>
-      <c r="W35" s="108"/>
-      <c r="X35" s="108"/>
-      <c r="Y35" s="108"/>
-      <c r="Z35" s="108"/>
-      <c r="AA35" s="108"/>
-      <c r="AB35" s="108"/>
-      <c r="AC35" s="108"/>
-      <c r="AD35" s="108"/>
-      <c r="AE35" s="108"/>
-      <c r="AF35" s="109"/>
-      <c r="AG35" s="105"/>
+      <c r="O35" s="158"/>
+      <c r="P35" s="158"/>
+      <c r="Q35" s="158"/>
+      <c r="R35" s="158"/>
+      <c r="S35" s="158"/>
+      <c r="T35" s="158"/>
+      <c r="U35" s="158"/>
+      <c r="V35" s="158"/>
+      <c r="W35" s="158"/>
+      <c r="X35" s="158"/>
+      <c r="Y35" s="158"/>
+      <c r="Z35" s="158"/>
+      <c r="AA35" s="158"/>
+      <c r="AB35" s="158"/>
+      <c r="AC35" s="158"/>
+      <c r="AD35" s="158"/>
+      <c r="AE35" s="158"/>
+      <c r="AF35" s="159"/>
+      <c r="AG35" s="155"/>
       <c r="AH35" s="13" t="s">
         <v>19</v>
       </c>
@@ -6605,88 +6605,88 @@
       <c r="AU36" s="2"/>
     </row>
     <row r="37" spans="1:54" ht="17" x14ac:dyDescent="0.2">
-      <c r="A37" s="115" t="s">
+      <c r="A37" s="151" t="s">
         <v>57</v>
       </c>
-      <c r="B37" s="116"/>
-      <c r="C37" s="116"/>
-      <c r="D37" s="116"/>
-      <c r="E37" s="116"/>
-      <c r="F37" s="116"/>
-      <c r="G37" s="116"/>
-      <c r="H37" s="116"/>
-      <c r="I37" s="116"/>
-      <c r="J37" s="116"/>
-      <c r="K37" s="116"/>
-      <c r="L37" s="116"/>
-      <c r="M37" s="116"/>
-      <c r="N37" s="116"/>
-      <c r="O37" s="116"/>
-      <c r="P37" s="116"/>
-      <c r="Q37" s="116"/>
-      <c r="R37" s="116"/>
-      <c r="S37" s="116"/>
-      <c r="T37" s="116"/>
-      <c r="U37" s="116"/>
-      <c r="V37" s="116"/>
-      <c r="W37" s="116"/>
-      <c r="X37" s="116"/>
-      <c r="Y37" s="116"/>
-      <c r="Z37" s="116"/>
-      <c r="AA37" s="116"/>
-      <c r="AB37" s="116"/>
-      <c r="AC37" s="116"/>
-      <c r="AD37" s="116"/>
-      <c r="AE37" s="116"/>
-      <c r="AF37" s="117"/>
+      <c r="B37" s="152"/>
+      <c r="C37" s="152"/>
+      <c r="D37" s="152"/>
+      <c r="E37" s="152"/>
+      <c r="F37" s="152"/>
+      <c r="G37" s="152"/>
+      <c r="H37" s="152"/>
+      <c r="I37" s="152"/>
+      <c r="J37" s="152"/>
+      <c r="K37" s="152"/>
+      <c r="L37" s="152"/>
+      <c r="M37" s="152"/>
+      <c r="N37" s="152"/>
+      <c r="O37" s="152"/>
+      <c r="P37" s="152"/>
+      <c r="Q37" s="152"/>
+      <c r="R37" s="152"/>
+      <c r="S37" s="152"/>
+      <c r="T37" s="152"/>
+      <c r="U37" s="152"/>
+      <c r="V37" s="152"/>
+      <c r="W37" s="152"/>
+      <c r="X37" s="152"/>
+      <c r="Y37" s="152"/>
+      <c r="Z37" s="152"/>
+      <c r="AA37" s="152"/>
+      <c r="AB37" s="152"/>
+      <c r="AC37" s="152"/>
+      <c r="AD37" s="152"/>
+      <c r="AE37" s="152"/>
+      <c r="AF37" s="153"/>
       <c r="AH37" s="20"/>
     </row>
     <row r="38" spans="1:54" x14ac:dyDescent="0.2">
-      <c r="A38" s="150" t="s">
+      <c r="A38" s="112" t="s">
         <v>58</v>
       </c>
-      <c r="B38" s="151"/>
-      <c r="C38" s="151"/>
-      <c r="D38" s="151"/>
-      <c r="E38" s="152">
+      <c r="B38" s="113"/>
+      <c r="C38" s="113"/>
+      <c r="D38" s="113"/>
+      <c r="E38" s="114">
         <v>40</v>
       </c>
-      <c r="F38" s="152"/>
-      <c r="G38" s="152"/>
-      <c r="H38" s="151" t="s">
+      <c r="F38" s="114"/>
+      <c r="G38" s="114"/>
+      <c r="H38" s="113" t="s">
         <v>59</v>
       </c>
-      <c r="I38" s="151"/>
-      <c r="J38" s="151"/>
-      <c r="K38" s="151"/>
-      <c r="L38" s="151"/>
-      <c r="M38" s="153"/>
-      <c r="N38" s="149" t="s">
+      <c r="I38" s="113"/>
+      <c r="J38" s="113"/>
+      <c r="K38" s="113"/>
+      <c r="L38" s="113"/>
+      <c r="M38" s="115"/>
+      <c r="N38" s="111" t="s">
         <v>60</v>
       </c>
-      <c r="O38" s="149"/>
-      <c r="P38" s="149"/>
-      <c r="Q38" s="149"/>
-      <c r="R38" s="149"/>
-      <c r="S38" s="149"/>
-      <c r="T38" s="149"/>
-      <c r="U38" s="149"/>
-      <c r="V38" s="149"/>
-      <c r="W38" s="149"/>
-      <c r="X38" s="149"/>
-      <c r="Y38" s="149"/>
-      <c r="Z38" s="149"/>
-      <c r="AA38" s="121">
+      <c r="O38" s="111"/>
+      <c r="P38" s="111"/>
+      <c r="Q38" s="111"/>
+      <c r="R38" s="111"/>
+      <c r="S38" s="111"/>
+      <c r="T38" s="111"/>
+      <c r="U38" s="111"/>
+      <c r="V38" s="111"/>
+      <c r="W38" s="111"/>
+      <c r="X38" s="111"/>
+      <c r="Y38" s="111"/>
+      <c r="Z38" s="111"/>
+      <c r="AA38" s="119">
         <f>$E$38*52</f>
         <v>2080</v>
       </c>
-      <c r="AB38" s="122"/>
-      <c r="AC38" s="123"/>
-      <c r="AD38" s="118" t="s">
+      <c r="AB38" s="120"/>
+      <c r="AC38" s="121"/>
+      <c r="AD38" s="122" t="s">
         <v>59</v>
       </c>
-      <c r="AE38" s="119"/>
-      <c r="AF38" s="120"/>
+      <c r="AE38" s="123"/>
+      <c r="AF38" s="124"/>
       <c r="AG38" s="37"/>
       <c r="AH38" s="21"/>
       <c r="AI38" s="2"/>
@@ -6696,53 +6696,53 @@
       <c r="A39" s="28" t="s">
         <v>61</v>
       </c>
-      <c r="B39" s="170" t="s">
+      <c r="B39" s="94" t="s">
         <v>62</v>
       </c>
-      <c r="C39" s="171"/>
-      <c r="D39" s="171"/>
-      <c r="E39" s="171"/>
-      <c r="F39" s="171"/>
-      <c r="G39" s="171"/>
-      <c r="H39" s="171"/>
-      <c r="I39" s="171"/>
-      <c r="J39" s="171"/>
-      <c r="K39" s="171"/>
-      <c r="L39" s="171"/>
-      <c r="M39" s="171"/>
-      <c r="N39" s="172"/>
-      <c r="O39" s="186">
+      <c r="C39" s="95"/>
+      <c r="D39" s="95"/>
+      <c r="E39" s="95"/>
+      <c r="F39" s="95"/>
+      <c r="G39" s="95"/>
+      <c r="H39" s="95"/>
+      <c r="I39" s="95"/>
+      <c r="J39" s="95"/>
+      <c r="K39" s="95"/>
+      <c r="L39" s="95"/>
+      <c r="M39" s="95"/>
+      <c r="N39" s="96"/>
+      <c r="O39" s="101">
         <v>30</v>
       </c>
-      <c r="P39" s="187"/>
-      <c r="Q39" s="188"/>
-      <c r="R39" s="124" t="s">
+      <c r="P39" s="102"/>
+      <c r="Q39" s="103"/>
+      <c r="R39" s="88" t="s">
         <v>63</v>
       </c>
-      <c r="S39" s="125"/>
-      <c r="T39" s="126"/>
-      <c r="U39" s="127">
+      <c r="S39" s="89"/>
+      <c r="T39" s="90"/>
+      <c r="U39" s="91">
         <f>$E$38/5</f>
         <v>8</v>
       </c>
-      <c r="V39" s="128"/>
-      <c r="W39" s="129"/>
-      <c r="X39" s="124" t="s">
+      <c r="V39" s="92"/>
+      <c r="W39" s="93"/>
+      <c r="X39" s="88" t="s">
         <v>64</v>
       </c>
-      <c r="Y39" s="125"/>
-      <c r="Z39" s="126"/>
-      <c r="AA39" s="121">
+      <c r="Y39" s="89"/>
+      <c r="Z39" s="90"/>
+      <c r="AA39" s="119">
         <f>U39*O39</f>
         <v>240</v>
       </c>
-      <c r="AB39" s="122"/>
-      <c r="AC39" s="123"/>
-      <c r="AD39" s="118" t="s">
+      <c r="AB39" s="120"/>
+      <c r="AC39" s="121"/>
+      <c r="AD39" s="122" t="s">
         <v>59</v>
       </c>
-      <c r="AE39" s="119"/>
-      <c r="AF39" s="120"/>
+      <c r="AE39" s="123"/>
+      <c r="AF39" s="124"/>
       <c r="AG39" s="37"/>
       <c r="AH39" s="21"/>
       <c r="AK39" s="1"/>
@@ -6780,53 +6780,53 @@
     </row>
     <row r="40" spans="1:54" s="2" customFormat="1" ht="16.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A40" s="29"/>
-      <c r="B40" s="170" t="s">
+      <c r="B40" s="94" t="s">
         <v>72</v>
       </c>
-      <c r="C40" s="171"/>
-      <c r="D40" s="171"/>
-      <c r="E40" s="171"/>
-      <c r="F40" s="171"/>
-      <c r="G40" s="171"/>
-      <c r="H40" s="171"/>
-      <c r="I40" s="171"/>
-      <c r="J40" s="171"/>
-      <c r="K40" s="171"/>
-      <c r="L40" s="171"/>
-      <c r="M40" s="171"/>
-      <c r="N40" s="172"/>
-      <c r="O40" s="130">
+      <c r="C40" s="95"/>
+      <c r="D40" s="95"/>
+      <c r="E40" s="95"/>
+      <c r="F40" s="95"/>
+      <c r="G40" s="95"/>
+      <c r="H40" s="95"/>
+      <c r="I40" s="95"/>
+      <c r="J40" s="95"/>
+      <c r="K40" s="95"/>
+      <c r="L40" s="95"/>
+      <c r="M40" s="95"/>
+      <c r="N40" s="96"/>
+      <c r="O40" s="104">
         <v>0</v>
       </c>
-      <c r="P40" s="131"/>
-      <c r="Q40" s="132"/>
-      <c r="R40" s="124" t="s">
+      <c r="P40" s="105"/>
+      <c r="Q40" s="106"/>
+      <c r="R40" s="88" t="s">
         <v>63</v>
       </c>
-      <c r="S40" s="125"/>
-      <c r="T40" s="126"/>
-      <c r="U40" s="127">
+      <c r="S40" s="89"/>
+      <c r="T40" s="90"/>
+      <c r="U40" s="91">
         <f t="shared" ref="U40:U43" si="41">$E$38/5</f>
         <v>8</v>
       </c>
-      <c r="V40" s="128"/>
-      <c r="W40" s="129"/>
-      <c r="X40" s="124" t="s">
+      <c r="V40" s="92"/>
+      <c r="W40" s="93"/>
+      <c r="X40" s="88" t="s">
         <v>64</v>
       </c>
-      <c r="Y40" s="125"/>
-      <c r="Z40" s="126"/>
-      <c r="AA40" s="121">
+      <c r="Y40" s="89"/>
+      <c r="Z40" s="90"/>
+      <c r="AA40" s="119">
         <f t="shared" ref="AA40:AA43" si="42">U40*O40</f>
         <v>0</v>
       </c>
-      <c r="AB40" s="122"/>
-      <c r="AC40" s="123"/>
-      <c r="AD40" s="118" t="s">
+      <c r="AB40" s="120"/>
+      <c r="AC40" s="121"/>
+      <c r="AD40" s="122" t="s">
         <v>59</v>
       </c>
-      <c r="AE40" s="119"/>
-      <c r="AF40" s="120"/>
+      <c r="AE40" s="123"/>
+      <c r="AF40" s="124"/>
       <c r="AG40" s="37"/>
       <c r="AH40" s="21"/>
       <c r="AK40" s="37"/>
@@ -6862,53 +6862,53 @@
     </row>
     <row r="41" spans="1:54" s="2" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A41" s="29"/>
-      <c r="B41" s="170" t="s">
+      <c r="B41" s="94" t="s">
         <v>75</v>
       </c>
-      <c r="C41" s="171"/>
-      <c r="D41" s="171"/>
-      <c r="E41" s="171"/>
-      <c r="F41" s="171"/>
-      <c r="G41" s="171"/>
-      <c r="H41" s="171"/>
-      <c r="I41" s="171"/>
-      <c r="J41" s="171"/>
-      <c r="K41" s="171"/>
-      <c r="L41" s="171"/>
-      <c r="M41" s="171"/>
-      <c r="N41" s="172"/>
-      <c r="O41" s="130">
+      <c r="C41" s="95"/>
+      <c r="D41" s="95"/>
+      <c r="E41" s="95"/>
+      <c r="F41" s="95"/>
+      <c r="G41" s="95"/>
+      <c r="H41" s="95"/>
+      <c r="I41" s="95"/>
+      <c r="J41" s="95"/>
+      <c r="K41" s="95"/>
+      <c r="L41" s="95"/>
+      <c r="M41" s="95"/>
+      <c r="N41" s="96"/>
+      <c r="O41" s="104">
         <v>0</v>
       </c>
-      <c r="P41" s="131"/>
-      <c r="Q41" s="132"/>
-      <c r="R41" s="124" t="s">
+      <c r="P41" s="105"/>
+      <c r="Q41" s="106"/>
+      <c r="R41" s="88" t="s">
         <v>63</v>
       </c>
-      <c r="S41" s="125"/>
-      <c r="T41" s="126"/>
-      <c r="U41" s="127">
+      <c r="S41" s="89"/>
+      <c r="T41" s="90"/>
+      <c r="U41" s="91">
         <f t="shared" si="41"/>
         <v>8</v>
       </c>
-      <c r="V41" s="128"/>
-      <c r="W41" s="129"/>
-      <c r="X41" s="124" t="s">
+      <c r="V41" s="92"/>
+      <c r="W41" s="93"/>
+      <c r="X41" s="88" t="s">
         <v>64</v>
       </c>
-      <c r="Y41" s="125"/>
-      <c r="Z41" s="126"/>
-      <c r="AA41" s="121">
+      <c r="Y41" s="89"/>
+      <c r="Z41" s="90"/>
+      <c r="AA41" s="119">
         <f t="shared" si="42"/>
         <v>0</v>
       </c>
-      <c r="AB41" s="122"/>
-      <c r="AC41" s="123"/>
-      <c r="AD41" s="118" t="s">
+      <c r="AB41" s="120"/>
+      <c r="AC41" s="121"/>
+      <c r="AD41" s="122" t="s">
         <v>59</v>
       </c>
-      <c r="AE41" s="119"/>
-      <c r="AF41" s="120"/>
+      <c r="AE41" s="123"/>
+      <c r="AF41" s="124"/>
       <c r="AG41" s="37"/>
       <c r="AH41" s="21"/>
       <c r="AK41" s="37"/>
@@ -6936,54 +6936,54 @@
     </row>
     <row r="42" spans="1:54" s="2" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A42" s="29"/>
-      <c r="B42" s="170" t="s">
+      <c r="B42" s="94" t="s">
         <v>77</v>
       </c>
-      <c r="C42" s="171"/>
-      <c r="D42" s="171"/>
-      <c r="E42" s="171"/>
-      <c r="F42" s="171"/>
-      <c r="G42" s="171"/>
-      <c r="H42" s="171"/>
-      <c r="I42" s="171"/>
-      <c r="J42" s="171"/>
-      <c r="K42" s="171"/>
-      <c r="L42" s="171"/>
-      <c r="M42" s="171"/>
-      <c r="N42" s="172"/>
-      <c r="O42" s="182">
+      <c r="C42" s="95"/>
+      <c r="D42" s="95"/>
+      <c r="E42" s="95"/>
+      <c r="F42" s="95"/>
+      <c r="G42" s="95"/>
+      <c r="H42" s="95"/>
+      <c r="I42" s="95"/>
+      <c r="J42" s="95"/>
+      <c r="K42" s="95"/>
+      <c r="L42" s="95"/>
+      <c r="M42" s="95"/>
+      <c r="N42" s="96"/>
+      <c r="O42" s="97">
         <f>AZ30</f>
         <v>9</v>
       </c>
-      <c r="P42" s="183"/>
-      <c r="Q42" s="184"/>
-      <c r="R42" s="124" t="s">
+      <c r="P42" s="98"/>
+      <c r="Q42" s="99"/>
+      <c r="R42" s="88" t="s">
         <v>63</v>
       </c>
-      <c r="S42" s="125"/>
-      <c r="T42" s="126"/>
-      <c r="U42" s="127">
+      <c r="S42" s="89"/>
+      <c r="T42" s="90"/>
+      <c r="U42" s="91">
         <f t="shared" si="41"/>
         <v>8</v>
       </c>
-      <c r="V42" s="128"/>
-      <c r="W42" s="129"/>
-      <c r="X42" s="124" t="s">
+      <c r="V42" s="92"/>
+      <c r="W42" s="93"/>
+      <c r="X42" s="88" t="s">
         <v>64</v>
       </c>
-      <c r="Y42" s="125"/>
-      <c r="Z42" s="126"/>
-      <c r="AA42" s="121">
+      <c r="Y42" s="89"/>
+      <c r="Z42" s="90"/>
+      <c r="AA42" s="119">
         <f t="shared" si="42"/>
         <v>72</v>
       </c>
-      <c r="AB42" s="122"/>
-      <c r="AC42" s="123"/>
-      <c r="AD42" s="118" t="s">
+      <c r="AB42" s="120"/>
+      <c r="AC42" s="121"/>
+      <c r="AD42" s="122" t="s">
         <v>59</v>
       </c>
-      <c r="AE42" s="119"/>
-      <c r="AF42" s="120"/>
+      <c r="AE42" s="123"/>
+      <c r="AF42" s="124"/>
       <c r="AG42" s="37"/>
       <c r="AH42" s="21"/>
       <c r="AK42" s="37"/>
@@ -7005,53 +7005,53 @@
     </row>
     <row r="43" spans="1:54" s="2" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A43" s="30"/>
-      <c r="B43" s="170" t="s">
+      <c r="B43" s="94" t="s">
         <v>80</v>
       </c>
-      <c r="C43" s="171"/>
-      <c r="D43" s="171"/>
-      <c r="E43" s="171"/>
-      <c r="F43" s="171"/>
-      <c r="G43" s="171"/>
-      <c r="H43" s="171"/>
-      <c r="I43" s="171"/>
-      <c r="J43" s="171"/>
-      <c r="K43" s="171"/>
-      <c r="L43" s="171"/>
-      <c r="M43" s="171"/>
-      <c r="N43" s="172"/>
-      <c r="O43" s="130">
+      <c r="C43" s="95"/>
+      <c r="D43" s="95"/>
+      <c r="E43" s="95"/>
+      <c r="F43" s="95"/>
+      <c r="G43" s="95"/>
+      <c r="H43" s="95"/>
+      <c r="I43" s="95"/>
+      <c r="J43" s="95"/>
+      <c r="K43" s="95"/>
+      <c r="L43" s="95"/>
+      <c r="M43" s="95"/>
+      <c r="N43" s="96"/>
+      <c r="O43" s="104">
         <v>0</v>
       </c>
-      <c r="P43" s="131"/>
-      <c r="Q43" s="132"/>
-      <c r="R43" s="124" t="s">
+      <c r="P43" s="105"/>
+      <c r="Q43" s="106"/>
+      <c r="R43" s="88" t="s">
         <v>63</v>
       </c>
-      <c r="S43" s="125"/>
-      <c r="T43" s="126"/>
-      <c r="U43" s="127">
+      <c r="S43" s="89"/>
+      <c r="T43" s="90"/>
+      <c r="U43" s="91">
         <f t="shared" si="41"/>
         <v>8</v>
       </c>
-      <c r="V43" s="128"/>
-      <c r="W43" s="129"/>
-      <c r="X43" s="124" t="s">
+      <c r="V43" s="92"/>
+      <c r="W43" s="93"/>
+      <c r="X43" s="88" t="s">
         <v>64</v>
       </c>
-      <c r="Y43" s="125"/>
-      <c r="Z43" s="126"/>
-      <c r="AA43" s="121">
+      <c r="Y43" s="89"/>
+      <c r="Z43" s="90"/>
+      <c r="AA43" s="119">
         <f t="shared" si="42"/>
         <v>0</v>
       </c>
-      <c r="AB43" s="122"/>
-      <c r="AC43" s="123"/>
-      <c r="AD43" s="118" t="s">
+      <c r="AB43" s="120"/>
+      <c r="AC43" s="121"/>
+      <c r="AD43" s="122" t="s">
         <v>59</v>
       </c>
-      <c r="AE43" s="119"/>
-      <c r="AF43" s="120"/>
+      <c r="AE43" s="123"/>
+      <c r="AF43" s="124"/>
       <c r="AG43" s="37"/>
       <c r="AH43" s="21"/>
       <c r="AK43" s="37"/>
@@ -7075,44 +7075,44 @@
       <c r="A44" s="31" t="s">
         <v>82</v>
       </c>
-      <c r="B44" s="185" t="s">
+      <c r="B44" s="100" t="s">
         <v>83</v>
       </c>
-      <c r="C44" s="185"/>
-      <c r="D44" s="185"/>
-      <c r="E44" s="185"/>
-      <c r="F44" s="185"/>
-      <c r="G44" s="185"/>
-      <c r="H44" s="185"/>
-      <c r="I44" s="185"/>
-      <c r="J44" s="185"/>
-      <c r="K44" s="185"/>
-      <c r="L44" s="185"/>
-      <c r="M44" s="185"/>
-      <c r="N44" s="185"/>
-      <c r="O44" s="185"/>
-      <c r="P44" s="185"/>
-      <c r="Q44" s="185"/>
-      <c r="R44" s="185"/>
-      <c r="S44" s="185"/>
-      <c r="T44" s="185"/>
-      <c r="U44" s="185"/>
-      <c r="V44" s="185"/>
-      <c r="W44" s="185"/>
-      <c r="X44" s="185"/>
-      <c r="Y44" s="185"/>
-      <c r="Z44" s="185"/>
-      <c r="AA44" s="139">
+      <c r="C44" s="100"/>
+      <c r="D44" s="100"/>
+      <c r="E44" s="100"/>
+      <c r="F44" s="100"/>
+      <c r="G44" s="100"/>
+      <c r="H44" s="100"/>
+      <c r="I44" s="100"/>
+      <c r="J44" s="100"/>
+      <c r="K44" s="100"/>
+      <c r="L44" s="100"/>
+      <c r="M44" s="100"/>
+      <c r="N44" s="100"/>
+      <c r="O44" s="100"/>
+      <c r="P44" s="100"/>
+      <c r="Q44" s="100"/>
+      <c r="R44" s="100"/>
+      <c r="S44" s="100"/>
+      <c r="T44" s="100"/>
+      <c r="U44" s="100"/>
+      <c r="V44" s="100"/>
+      <c r="W44" s="100"/>
+      <c r="X44" s="100"/>
+      <c r="Y44" s="100"/>
+      <c r="Z44" s="100"/>
+      <c r="AA44" s="144">
         <f>AA38-SUM(AA39:AC43)</f>
         <v>1768</v>
       </c>
-      <c r="AB44" s="140"/>
-      <c r="AC44" s="141"/>
-      <c r="AD44" s="133" t="s">
+      <c r="AB44" s="145"/>
+      <c r="AC44" s="146"/>
+      <c r="AD44" s="138" t="s">
         <v>59</v>
       </c>
-      <c r="AE44" s="134"/>
-      <c r="AF44" s="135"/>
+      <c r="AE44" s="139"/>
+      <c r="AF44" s="140"/>
       <c r="AG44" s="37"/>
       <c r="AH44" s="21"/>
       <c r="AK44" s="37"/>
@@ -7133,48 +7133,48 @@
       <c r="BA44" s="74"/>
     </row>
     <row r="45" spans="1:54" s="2" customFormat="1" ht="16" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A45" s="157" t="s">
+      <c r="A45" s="125" t="s">
         <v>86</v>
       </c>
-      <c r="B45" s="158"/>
-      <c r="C45" s="158"/>
-      <c r="D45" s="158"/>
-      <c r="E45" s="158"/>
-      <c r="F45" s="158"/>
-      <c r="G45" s="158"/>
-      <c r="H45" s="158"/>
-      <c r="I45" s="158"/>
-      <c r="J45" s="158"/>
-      <c r="K45" s="158"/>
-      <c r="L45" s="158"/>
-      <c r="M45" s="158"/>
-      <c r="N45" s="158"/>
-      <c r="O45" s="158"/>
-      <c r="P45" s="158"/>
-      <c r="Q45" s="158"/>
-      <c r="R45" s="158"/>
-      <c r="S45" s="158"/>
-      <c r="T45" s="158"/>
-      <c r="U45" s="158"/>
-      <c r="V45" s="158"/>
-      <c r="W45" s="159"/>
-      <c r="X45" s="160">
+      <c r="B45" s="126"/>
+      <c r="C45" s="126"/>
+      <c r="D45" s="126"/>
+      <c r="E45" s="126"/>
+      <c r="F45" s="126"/>
+      <c r="G45" s="126"/>
+      <c r="H45" s="126"/>
+      <c r="I45" s="126"/>
+      <c r="J45" s="126"/>
+      <c r="K45" s="126"/>
+      <c r="L45" s="126"/>
+      <c r="M45" s="126"/>
+      <c r="N45" s="126"/>
+      <c r="O45" s="126"/>
+      <c r="P45" s="126"/>
+      <c r="Q45" s="126"/>
+      <c r="R45" s="126"/>
+      <c r="S45" s="126"/>
+      <c r="T45" s="126"/>
+      <c r="U45" s="126"/>
+      <c r="V45" s="126"/>
+      <c r="W45" s="127"/>
+      <c r="X45" s="128">
         <f>1/12*5</f>
         <v>0.41666666666666663</v>
       </c>
-      <c r="Y45" s="161"/>
-      <c r="Z45" s="162"/>
-      <c r="AA45" s="142">
+      <c r="Y45" s="129"/>
+      <c r="Z45" s="130"/>
+      <c r="AA45" s="147">
         <f>AA44*X45</f>
         <v>736.66666666666663</v>
       </c>
-      <c r="AB45" s="143"/>
-      <c r="AC45" s="144"/>
-      <c r="AD45" s="136" t="s">
+      <c r="AB45" s="148"/>
+      <c r="AC45" s="149"/>
+      <c r="AD45" s="141" t="s">
         <v>59</v>
       </c>
-      <c r="AE45" s="137"/>
-      <c r="AF45" s="138"/>
+      <c r="AE45" s="142"/>
+      <c r="AF45" s="143"/>
       <c r="AG45" s="24"/>
       <c r="AH45" s="25"/>
       <c r="AI45" s="23"/>
@@ -7259,28 +7259,28 @@
       <c r="BB46" s="2"/>
     </row>
     <row r="47" spans="1:54" s="2" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A47" s="154" t="s">
+      <c r="A47" s="116" t="s">
         <v>91</v>
       </c>
-      <c r="B47" s="155"/>
-      <c r="C47" s="155"/>
-      <c r="D47" s="155"/>
-      <c r="E47" s="155"/>
-      <c r="F47" s="155"/>
-      <c r="G47" s="155"/>
-      <c r="H47" s="155"/>
-      <c r="I47" s="155"/>
-      <c r="J47" s="155"/>
-      <c r="K47" s="155"/>
-      <c r="L47" s="155"/>
-      <c r="M47" s="155"/>
-      <c r="N47" s="155"/>
-      <c r="O47" s="155"/>
-      <c r="P47" s="155"/>
-      <c r="Q47" s="155"/>
-      <c r="R47" s="155"/>
-      <c r="S47" s="155"/>
-      <c r="T47" s="156"/>
+      <c r="B47" s="117"/>
+      <c r="C47" s="117"/>
+      <c r="D47" s="117"/>
+      <c r="E47" s="117"/>
+      <c r="F47" s="117"/>
+      <c r="G47" s="117"/>
+      <c r="H47" s="117"/>
+      <c r="I47" s="117"/>
+      <c r="J47" s="117"/>
+      <c r="K47" s="117"/>
+      <c r="L47" s="117"/>
+      <c r="M47" s="117"/>
+      <c r="N47" s="117"/>
+      <c r="O47" s="117"/>
+      <c r="P47" s="117"/>
+      <c r="Q47" s="117"/>
+      <c r="R47" s="117"/>
+      <c r="S47" s="117"/>
+      <c r="T47" s="118"/>
       <c r="U47" s="37"/>
       <c r="V47" s="21"/>
       <c r="AK47" s="24"/>
@@ -7303,33 +7303,33 @@
       <c r="BA47" s="74"/>
     </row>
     <row r="48" spans="1:54" s="2" customFormat="1" ht="17" x14ac:dyDescent="0.2">
-      <c r="A48" s="150" t="s">
+      <c r="A48" s="112" t="s">
         <v>94</v>
       </c>
-      <c r="B48" s="151"/>
-      <c r="C48" s="151"/>
-      <c r="D48" s="151"/>
-      <c r="E48" s="151"/>
-      <c r="F48" s="151"/>
-      <c r="G48" s="151"/>
-      <c r="H48" s="151"/>
-      <c r="I48" s="151"/>
-      <c r="J48" s="151"/>
-      <c r="K48" s="151"/>
-      <c r="L48" s="151"/>
-      <c r="M48" s="151"/>
-      <c r="N48" s="151"/>
-      <c r="O48" s="121">
+      <c r="B48" s="113"/>
+      <c r="C48" s="113"/>
+      <c r="D48" s="113"/>
+      <c r="E48" s="113"/>
+      <c r="F48" s="113"/>
+      <c r="G48" s="113"/>
+      <c r="H48" s="113"/>
+      <c r="I48" s="113"/>
+      <c r="J48" s="113"/>
+      <c r="K48" s="113"/>
+      <c r="L48" s="113"/>
+      <c r="M48" s="113"/>
+      <c r="N48" s="113"/>
+      <c r="O48" s="119">
         <f>AG34</f>
         <v>297</v>
       </c>
-      <c r="P48" s="122"/>
-      <c r="Q48" s="123"/>
-      <c r="R48" s="118" t="s">
+      <c r="P48" s="120"/>
+      <c r="Q48" s="121"/>
+      <c r="R48" s="122" t="s">
         <v>59</v>
       </c>
-      <c r="S48" s="119"/>
-      <c r="T48" s="120"/>
+      <c r="S48" s="123"/>
+      <c r="T48" s="124"/>
       <c r="U48" s="37"/>
       <c r="V48" s="21"/>
       <c r="AK48" s="37"/>
@@ -7361,32 +7361,32 @@
       <c r="A49" s="26" t="s">
         <v>97</v>
       </c>
-      <c r="B49" s="170" t="s">
+      <c r="B49" s="94" t="s">
         <v>98</v>
       </c>
-      <c r="C49" s="171"/>
-      <c r="D49" s="171"/>
-      <c r="E49" s="171"/>
-      <c r="F49" s="171"/>
-      <c r="G49" s="171"/>
-      <c r="H49" s="171"/>
-      <c r="I49" s="171"/>
-      <c r="J49" s="171"/>
-      <c r="K49" s="171"/>
-      <c r="L49" s="171"/>
-      <c r="M49" s="171"/>
-      <c r="N49" s="172"/>
-      <c r="O49" s="163">
+      <c r="C49" s="95"/>
+      <c r="D49" s="95"/>
+      <c r="E49" s="95"/>
+      <c r="F49" s="95"/>
+      <c r="G49" s="95"/>
+      <c r="H49" s="95"/>
+      <c r="I49" s="95"/>
+      <c r="J49" s="95"/>
+      <c r="K49" s="95"/>
+      <c r="L49" s="95"/>
+      <c r="M49" s="95"/>
+      <c r="N49" s="96"/>
+      <c r="O49" s="131">
         <f>AA45</f>
         <v>736.66666666666663</v>
       </c>
-      <c r="P49" s="164"/>
-      <c r="Q49" s="165"/>
-      <c r="R49" s="118" t="s">
+      <c r="P49" s="132"/>
+      <c r="Q49" s="133"/>
+      <c r="R49" s="122" t="s">
         <v>59</v>
       </c>
-      <c r="S49" s="119"/>
-      <c r="T49" s="120"/>
+      <c r="S49" s="123"/>
+      <c r="T49" s="124"/>
       <c r="U49" s="37"/>
       <c r="V49" s="21"/>
       <c r="AK49" s="37"/>
@@ -7412,30 +7412,30 @@
       <c r="A50" s="27" t="s">
         <v>82</v>
       </c>
-      <c r="B50" s="166" t="s">
+      <c r="B50" s="134" t="s">
         <v>101</v>
       </c>
-      <c r="C50" s="166"/>
-      <c r="D50" s="166"/>
-      <c r="E50" s="166"/>
-      <c r="F50" s="166"/>
-      <c r="G50" s="166"/>
-      <c r="H50" s="166"/>
-      <c r="I50" s="166"/>
-      <c r="J50" s="166"/>
-      <c r="K50" s="166"/>
-      <c r="L50" s="166"/>
-      <c r="M50" s="166"/>
-      <c r="N50" s="166"/>
-      <c r="O50" s="167">
+      <c r="C50" s="134"/>
+      <c r="D50" s="134"/>
+      <c r="E50" s="134"/>
+      <c r="F50" s="134"/>
+      <c r="G50" s="134"/>
+      <c r="H50" s="134"/>
+      <c r="I50" s="134"/>
+      <c r="J50" s="134"/>
+      <c r="K50" s="134"/>
+      <c r="L50" s="134"/>
+      <c r="M50" s="134"/>
+      <c r="N50" s="134"/>
+      <c r="O50" s="135">
         <f>IF(O49=0,"-",O48/O49)</f>
         <v>0.40316742081447965</v>
       </c>
-      <c r="P50" s="168"/>
-      <c r="Q50" s="168"/>
-      <c r="R50" s="168"/>
-      <c r="S50" s="168"/>
-      <c r="T50" s="169"/>
+      <c r="P50" s="136"/>
+      <c r="Q50" s="136"/>
+      <c r="R50" s="136"/>
+      <c r="S50" s="136"/>
+      <c r="T50" s="137"/>
       <c r="AG50" s="37"/>
       <c r="AH50" s="21"/>
       <c r="AK50" s="37"/>
@@ -7482,28 +7482,28 @@
       <c r="BA51" s="74"/>
     </row>
     <row r="52" spans="1:53" s="2" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A52" s="154" t="s">
+      <c r="A52" s="116" t="s">
         <v>106</v>
       </c>
-      <c r="B52" s="155"/>
-      <c r="C52" s="155"/>
-      <c r="D52" s="155"/>
-      <c r="E52" s="155"/>
-      <c r="F52" s="155"/>
-      <c r="G52" s="155"/>
-      <c r="H52" s="155"/>
-      <c r="I52" s="155"/>
-      <c r="J52" s="155"/>
-      <c r="K52" s="155"/>
-      <c r="L52" s="155"/>
-      <c r="M52" s="155"/>
-      <c r="N52" s="155"/>
-      <c r="O52" s="155"/>
-      <c r="P52" s="155"/>
-      <c r="Q52" s="155"/>
-      <c r="R52" s="155"/>
-      <c r="S52" s="155"/>
-      <c r="T52" s="156"/>
+      <c r="B52" s="117"/>
+      <c r="C52" s="117"/>
+      <c r="D52" s="117"/>
+      <c r="E52" s="117"/>
+      <c r="F52" s="117"/>
+      <c r="G52" s="117"/>
+      <c r="H52" s="117"/>
+      <c r="I52" s="117"/>
+      <c r="J52" s="117"/>
+      <c r="K52" s="117"/>
+      <c r="L52" s="117"/>
+      <c r="M52" s="117"/>
+      <c r="N52" s="117"/>
+      <c r="O52" s="117"/>
+      <c r="P52" s="117"/>
+      <c r="Q52" s="117"/>
+      <c r="R52" s="117"/>
+      <c r="S52" s="117"/>
+      <c r="T52" s="118"/>
       <c r="AG52" s="37"/>
       <c r="AH52" s="21"/>
       <c r="AK52" s="37"/>
@@ -7530,33 +7530,33 @@
       </c>
     </row>
     <row r="53" spans="1:53" s="2" customFormat="1" ht="17" x14ac:dyDescent="0.2">
-      <c r="A53" s="150" t="s">
+      <c r="A53" s="112" t="s">
         <v>109</v>
       </c>
-      <c r="B53" s="151"/>
-      <c r="C53" s="151"/>
-      <c r="D53" s="151"/>
-      <c r="E53" s="151"/>
-      <c r="F53" s="151"/>
-      <c r="G53" s="151"/>
-      <c r="H53" s="151"/>
-      <c r="I53" s="151"/>
-      <c r="J53" s="151"/>
-      <c r="K53" s="151"/>
-      <c r="L53" s="151"/>
-      <c r="M53" s="151"/>
-      <c r="N53" s="151"/>
-      <c r="O53" s="121">
+      <c r="B53" s="113"/>
+      <c r="C53" s="113"/>
+      <c r="D53" s="113"/>
+      <c r="E53" s="113"/>
+      <c r="F53" s="113"/>
+      <c r="G53" s="113"/>
+      <c r="H53" s="113"/>
+      <c r="I53" s="113"/>
+      <c r="J53" s="113"/>
+      <c r="K53" s="113"/>
+      <c r="L53" s="113"/>
+      <c r="M53" s="113"/>
+      <c r="N53" s="113"/>
+      <c r="O53" s="119">
         <f>$AG$34</f>
         <v>297</v>
       </c>
-      <c r="P53" s="122"/>
-      <c r="Q53" s="123"/>
-      <c r="R53" s="118" t="s">
+      <c r="P53" s="120"/>
+      <c r="Q53" s="121"/>
+      <c r="R53" s="122" t="s">
         <v>59</v>
       </c>
-      <c r="S53" s="119"/>
-      <c r="T53" s="120"/>
+      <c r="S53" s="123"/>
+      <c r="T53" s="124"/>
       <c r="AG53" s="37"/>
       <c r="AH53" s="21"/>
       <c r="AK53" s="37"/>
@@ -7579,33 +7579,33 @@
       <c r="BA53" s="74"/>
     </row>
     <row r="54" spans="1:53" s="2" customFormat="1" ht="16" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A54" s="179" t="s">
+      <c r="A54" s="85" t="s">
         <v>112</v>
       </c>
-      <c r="B54" s="180"/>
-      <c r="C54" s="180"/>
-      <c r="D54" s="180"/>
-      <c r="E54" s="180"/>
-      <c r="F54" s="180"/>
-      <c r="G54" s="180"/>
-      <c r="H54" s="180"/>
-      <c r="I54" s="180"/>
-      <c r="J54" s="180"/>
-      <c r="K54" s="180"/>
-      <c r="L54" s="180"/>
-      <c r="M54" s="180"/>
-      <c r="N54" s="181"/>
-      <c r="O54" s="173">
+      <c r="B54" s="86"/>
+      <c r="C54" s="86"/>
+      <c r="D54" s="86"/>
+      <c r="E54" s="86"/>
+      <c r="F54" s="86"/>
+      <c r="G54" s="86"/>
+      <c r="H54" s="86"/>
+      <c r="I54" s="86"/>
+      <c r="J54" s="86"/>
+      <c r="K54" s="86"/>
+      <c r="L54" s="86"/>
+      <c r="M54" s="86"/>
+      <c r="N54" s="87"/>
+      <c r="O54" s="79">
         <f>X45*2080</f>
         <v>866.66666666666663</v>
       </c>
-      <c r="P54" s="174"/>
-      <c r="Q54" s="175"/>
-      <c r="R54" s="176" t="s">
+      <c r="P54" s="80"/>
+      <c r="Q54" s="81"/>
+      <c r="R54" s="82" t="s">
         <v>59</v>
       </c>
-      <c r="S54" s="177"/>
-      <c r="T54" s="178"/>
+      <c r="S54" s="83"/>
+      <c r="T54" s="84"/>
       <c r="AG54" s="37"/>
       <c r="AH54" s="21"/>
       <c r="AK54" s="37"/>
@@ -7661,23 +7661,23 @@
       <c r="I56" s="33"/>
       <c r="J56" s="33"/>
       <c r="K56" s="33"/>
-      <c r="T56" s="148" t="s">
+      <c r="T56" s="110" t="s">
         <v>116</v>
       </c>
-      <c r="U56" s="148"/>
-      <c r="V56" s="148"/>
-      <c r="W56" s="148"/>
-      <c r="X56" s="148"/>
-      <c r="Y56" s="148"/>
-      <c r="Z56" s="146"/>
-      <c r="AA56" s="146"/>
-      <c r="AB56" s="146"/>
-      <c r="AC56" s="146"/>
-      <c r="AD56" s="146"/>
-      <c r="AE56" s="146"/>
-      <c r="AF56" s="146"/>
-      <c r="AG56" s="146"/>
-      <c r="AH56" s="146"/>
+      <c r="U56" s="110"/>
+      <c r="V56" s="110"/>
+      <c r="W56" s="110"/>
+      <c r="X56" s="110"/>
+      <c r="Y56" s="110"/>
+      <c r="Z56" s="108"/>
+      <c r="AA56" s="108"/>
+      <c r="AB56" s="108"/>
+      <c r="AC56" s="108"/>
+      <c r="AD56" s="108"/>
+      <c r="AE56" s="108"/>
+      <c r="AF56" s="108"/>
+      <c r="AG56" s="108"/>
+      <c r="AH56" s="108"/>
       <c r="AK56" s="37"/>
       <c r="AO56" s="37"/>
       <c r="AP56" s="37"/>
@@ -7698,21 +7698,21 @@
       <c r="I57" s="34"/>
       <c r="J57" s="34"/>
       <c r="K57" s="34"/>
-      <c r="T57" s="148"/>
-      <c r="U57" s="148"/>
-      <c r="V57" s="148"/>
-      <c r="W57" s="148"/>
-      <c r="X57" s="148"/>
-      <c r="Y57" s="148"/>
-      <c r="Z57" s="147"/>
-      <c r="AA57" s="147"/>
-      <c r="AB57" s="147"/>
-      <c r="AC57" s="147"/>
-      <c r="AD57" s="147"/>
-      <c r="AE57" s="147"/>
-      <c r="AF57" s="147"/>
-      <c r="AG57" s="147"/>
-      <c r="AH57" s="147"/>
+      <c r="T57" s="110"/>
+      <c r="U57" s="110"/>
+      <c r="V57" s="110"/>
+      <c r="W57" s="110"/>
+      <c r="X57" s="110"/>
+      <c r="Y57" s="110"/>
+      <c r="Z57" s="109"/>
+      <c r="AA57" s="109"/>
+      <c r="AB57" s="109"/>
+      <c r="AC57" s="109"/>
+      <c r="AD57" s="109"/>
+      <c r="AE57" s="109"/>
+      <c r="AF57" s="109"/>
+      <c r="AG57" s="109"/>
+      <c r="AH57" s="109"/>
       <c r="AK57" s="37"/>
       <c r="AO57" s="37"/>
       <c r="AP57" s="37"/>
@@ -7722,30 +7722,30 @@
       <c r="AW57" s="37"/>
     </row>
     <row r="58" spans="1:53" s="2" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A58" s="145" t="s">
+      <c r="A58" s="107" t="s">
         <v>117</v>
       </c>
-      <c r="B58" s="145"/>
-      <c r="C58" s="145"/>
-      <c r="D58" s="145"/>
-      <c r="E58" s="145"/>
-      <c r="F58" s="145"/>
-      <c r="G58" s="145"/>
-      <c r="H58" s="145"/>
-      <c r="I58" s="145"/>
-      <c r="J58" s="145"/>
-      <c r="K58" s="145"/>
-      <c r="Z58" s="145" t="s">
+      <c r="B58" s="107"/>
+      <c r="C58" s="107"/>
+      <c r="D58" s="107"/>
+      <c r="E58" s="107"/>
+      <c r="F58" s="107"/>
+      <c r="G58" s="107"/>
+      <c r="H58" s="107"/>
+      <c r="I58" s="107"/>
+      <c r="J58" s="107"/>
+      <c r="K58" s="107"/>
+      <c r="Z58" s="107" t="s">
         <v>118</v>
       </c>
-      <c r="AA58" s="145"/>
-      <c r="AB58" s="145"/>
-      <c r="AC58" s="145"/>
-      <c r="AD58" s="145"/>
-      <c r="AE58" s="145"/>
-      <c r="AF58" s="145"/>
-      <c r="AG58" s="145"/>
-      <c r="AH58" s="145"/>
+      <c r="AA58" s="107"/>
+      <c r="AB58" s="107"/>
+      <c r="AC58" s="107"/>
+      <c r="AD58" s="107"/>
+      <c r="AE58" s="107"/>
+      <c r="AF58" s="107"/>
+      <c r="AG58" s="107"/>
+      <c r="AH58" s="107"/>
       <c r="AK58" s="37"/>
       <c r="AO58" s="37"/>
       <c r="AP58" s="37"/>
@@ -7776,42 +7776,42 @@
       <c r="AW59" s="37"/>
     </row>
     <row r="60" spans="1:53" s="2" customFormat="1" ht="24.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A60" s="114" t="s">
+      <c r="A60" s="150" t="s">
         <v>119</v>
       </c>
-      <c r="B60" s="114"/>
-      <c r="C60" s="114"/>
-      <c r="D60" s="114"/>
-      <c r="E60" s="114"/>
-      <c r="F60" s="114"/>
-      <c r="G60" s="114"/>
-      <c r="H60" s="114"/>
-      <c r="I60" s="114"/>
-      <c r="J60" s="114"/>
-      <c r="K60" s="114"/>
-      <c r="L60" s="114"/>
-      <c r="M60" s="114"/>
-      <c r="N60" s="114"/>
-      <c r="O60" s="114"/>
-      <c r="P60" s="114"/>
-      <c r="Q60" s="114"/>
-      <c r="R60" s="114"/>
-      <c r="S60" s="114"/>
-      <c r="T60" s="114"/>
-      <c r="U60" s="114"/>
-      <c r="V60" s="114"/>
-      <c r="W60" s="114"/>
-      <c r="X60" s="114"/>
-      <c r="Y60" s="114"/>
-      <c r="Z60" s="114"/>
-      <c r="AA60" s="114"/>
-      <c r="AB60" s="114"/>
-      <c r="AC60" s="114"/>
-      <c r="AD60" s="114"/>
-      <c r="AE60" s="114"/>
-      <c r="AF60" s="114"/>
-      <c r="AG60" s="114"/>
-      <c r="AH60" s="114"/>
+      <c r="B60" s="150"/>
+      <c r="C60" s="150"/>
+      <c r="D60" s="150"/>
+      <c r="E60" s="150"/>
+      <c r="F60" s="150"/>
+      <c r="G60" s="150"/>
+      <c r="H60" s="150"/>
+      <c r="I60" s="150"/>
+      <c r="J60" s="150"/>
+      <c r="K60" s="150"/>
+      <c r="L60" s="150"/>
+      <c r="M60" s="150"/>
+      <c r="N60" s="150"/>
+      <c r="O60" s="150"/>
+      <c r="P60" s="150"/>
+      <c r="Q60" s="150"/>
+      <c r="R60" s="150"/>
+      <c r="S60" s="150"/>
+      <c r="T60" s="150"/>
+      <c r="U60" s="150"/>
+      <c r="V60" s="150"/>
+      <c r="W60" s="150"/>
+      <c r="X60" s="150"/>
+      <c r="Y60" s="150"/>
+      <c r="Z60" s="150"/>
+      <c r="AA60" s="150"/>
+      <c r="AB60" s="150"/>
+      <c r="AC60" s="150"/>
+      <c r="AD60" s="150"/>
+      <c r="AE60" s="150"/>
+      <c r="AF60" s="150"/>
+      <c r="AG60" s="150"/>
+      <c r="AH60" s="150"/>
       <c r="AK60" s="37"/>
       <c r="AO60" s="37"/>
       <c r="AP60" s="37"/>
@@ -7821,42 +7821,42 @@
       <c r="AW60" s="37"/>
     </row>
     <row r="61" spans="1:53" s="2" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A61" s="114" t="s">
+      <c r="A61" s="150" t="s">
         <v>120</v>
       </c>
-      <c r="B61" s="114"/>
-      <c r="C61" s="114"/>
-      <c r="D61" s="114"/>
-      <c r="E61" s="114"/>
-      <c r="F61" s="114"/>
-      <c r="G61" s="114"/>
-      <c r="H61" s="114"/>
-      <c r="I61" s="114"/>
-      <c r="J61" s="114"/>
-      <c r="K61" s="114"/>
-      <c r="L61" s="114"/>
-      <c r="M61" s="114"/>
-      <c r="N61" s="114"/>
-      <c r="O61" s="114"/>
-      <c r="P61" s="114"/>
-      <c r="Q61" s="114"/>
-      <c r="R61" s="114"/>
-      <c r="S61" s="114"/>
-      <c r="T61" s="114"/>
-      <c r="U61" s="114"/>
-      <c r="V61" s="114"/>
-      <c r="W61" s="114"/>
-      <c r="X61" s="114"/>
-      <c r="Y61" s="114"/>
-      <c r="Z61" s="114"/>
-      <c r="AA61" s="114"/>
-      <c r="AB61" s="114"/>
-      <c r="AC61" s="114"/>
-      <c r="AD61" s="114"/>
-      <c r="AE61" s="114"/>
-      <c r="AF61" s="114"/>
-      <c r="AG61" s="114"/>
-      <c r="AH61" s="114"/>
+      <c r="B61" s="150"/>
+      <c r="C61" s="150"/>
+      <c r="D61" s="150"/>
+      <c r="E61" s="150"/>
+      <c r="F61" s="150"/>
+      <c r="G61" s="150"/>
+      <c r="H61" s="150"/>
+      <c r="I61" s="150"/>
+      <c r="J61" s="150"/>
+      <c r="K61" s="150"/>
+      <c r="L61" s="150"/>
+      <c r="M61" s="150"/>
+      <c r="N61" s="150"/>
+      <c r="O61" s="150"/>
+      <c r="P61" s="150"/>
+      <c r="Q61" s="150"/>
+      <c r="R61" s="150"/>
+      <c r="S61" s="150"/>
+      <c r="T61" s="150"/>
+      <c r="U61" s="150"/>
+      <c r="V61" s="150"/>
+      <c r="W61" s="150"/>
+      <c r="X61" s="150"/>
+      <c r="Y61" s="150"/>
+      <c r="Z61" s="150"/>
+      <c r="AA61" s="150"/>
+      <c r="AB61" s="150"/>
+      <c r="AC61" s="150"/>
+      <c r="AD61" s="150"/>
+      <c r="AE61" s="150"/>
+      <c r="AF61" s="150"/>
+      <c r="AG61" s="150"/>
+      <c r="AH61" s="150"/>
       <c r="AK61" s="37"/>
       <c r="AO61" s="37"/>
       <c r="AP61" s="37"/>
@@ -7866,42 +7866,42 @@
       <c r="AW61" s="37"/>
     </row>
     <row r="62" spans="1:53" s="2" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A62" s="114" t="s">
+      <c r="A62" s="150" t="s">
         <v>121</v>
       </c>
-      <c r="B62" s="114"/>
-      <c r="C62" s="114"/>
-      <c r="D62" s="114"/>
-      <c r="E62" s="114"/>
-      <c r="F62" s="114"/>
-      <c r="G62" s="114"/>
-      <c r="H62" s="114"/>
-      <c r="I62" s="114"/>
-      <c r="J62" s="114"/>
-      <c r="K62" s="114"/>
-      <c r="L62" s="114"/>
-      <c r="M62" s="114"/>
-      <c r="N62" s="114"/>
-      <c r="O62" s="114"/>
-      <c r="P62" s="114"/>
-      <c r="Q62" s="114"/>
-      <c r="R62" s="114"/>
-      <c r="S62" s="114"/>
-      <c r="T62" s="114"/>
-      <c r="U62" s="114"/>
-      <c r="V62" s="114"/>
-      <c r="W62" s="114"/>
-      <c r="X62" s="114"/>
-      <c r="Y62" s="114"/>
-      <c r="Z62" s="114"/>
-      <c r="AA62" s="114"/>
-      <c r="AB62" s="114"/>
-      <c r="AC62" s="114"/>
-      <c r="AD62" s="114"/>
-      <c r="AE62" s="114"/>
-      <c r="AF62" s="114"/>
-      <c r="AG62" s="114"/>
-      <c r="AH62" s="114"/>
+      <c r="B62" s="150"/>
+      <c r="C62" s="150"/>
+      <c r="D62" s="150"/>
+      <c r="E62" s="150"/>
+      <c r="F62" s="150"/>
+      <c r="G62" s="150"/>
+      <c r="H62" s="150"/>
+      <c r="I62" s="150"/>
+      <c r="J62" s="150"/>
+      <c r="K62" s="150"/>
+      <c r="L62" s="150"/>
+      <c r="M62" s="150"/>
+      <c r="N62" s="150"/>
+      <c r="O62" s="150"/>
+      <c r="P62" s="150"/>
+      <c r="Q62" s="150"/>
+      <c r="R62" s="150"/>
+      <c r="S62" s="150"/>
+      <c r="T62" s="150"/>
+      <c r="U62" s="150"/>
+      <c r="V62" s="150"/>
+      <c r="W62" s="150"/>
+      <c r="X62" s="150"/>
+      <c r="Y62" s="150"/>
+      <c r="Z62" s="150"/>
+      <c r="AA62" s="150"/>
+      <c r="AB62" s="150"/>
+      <c r="AC62" s="150"/>
+      <c r="AD62" s="150"/>
+      <c r="AE62" s="150"/>
+      <c r="AF62" s="150"/>
+      <c r="AG62" s="150"/>
+      <c r="AH62" s="150"/>
       <c r="AK62" s="37"/>
       <c r="AO62" s="37"/>
       <c r="AP62" s="37"/>
@@ -7911,42 +7911,42 @@
       <c r="AW62" s="37"/>
     </row>
     <row r="63" spans="1:53" s="2" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A63" s="114" t="s">
+      <c r="A63" s="150" t="s">
         <v>122</v>
       </c>
-      <c r="B63" s="114"/>
-      <c r="C63" s="114"/>
-      <c r="D63" s="114"/>
-      <c r="E63" s="114"/>
-      <c r="F63" s="114"/>
-      <c r="G63" s="114"/>
-      <c r="H63" s="114"/>
-      <c r="I63" s="114"/>
-      <c r="J63" s="114"/>
-      <c r="K63" s="114"/>
-      <c r="L63" s="114"/>
-      <c r="M63" s="114"/>
-      <c r="N63" s="114"/>
-      <c r="O63" s="114"/>
-      <c r="P63" s="114"/>
-      <c r="Q63" s="114"/>
-      <c r="R63" s="114"/>
-      <c r="S63" s="114"/>
-      <c r="T63" s="114"/>
-      <c r="U63" s="114"/>
-      <c r="V63" s="114"/>
-      <c r="W63" s="114"/>
-      <c r="X63" s="114"/>
-      <c r="Y63" s="114"/>
-      <c r="Z63" s="114"/>
-      <c r="AA63" s="114"/>
-      <c r="AB63" s="114"/>
-      <c r="AC63" s="114"/>
-      <c r="AD63" s="114"/>
-      <c r="AE63" s="114"/>
-      <c r="AF63" s="114"/>
-      <c r="AG63" s="114"/>
-      <c r="AH63" s="114"/>
+      <c r="B63" s="150"/>
+      <c r="C63" s="150"/>
+      <c r="D63" s="150"/>
+      <c r="E63" s="150"/>
+      <c r="F63" s="150"/>
+      <c r="G63" s="150"/>
+      <c r="H63" s="150"/>
+      <c r="I63" s="150"/>
+      <c r="J63" s="150"/>
+      <c r="K63" s="150"/>
+      <c r="L63" s="150"/>
+      <c r="M63" s="150"/>
+      <c r="N63" s="150"/>
+      <c r="O63" s="150"/>
+      <c r="P63" s="150"/>
+      <c r="Q63" s="150"/>
+      <c r="R63" s="150"/>
+      <c r="S63" s="150"/>
+      <c r="T63" s="150"/>
+      <c r="U63" s="150"/>
+      <c r="V63" s="150"/>
+      <c r="W63" s="150"/>
+      <c r="X63" s="150"/>
+      <c r="Y63" s="150"/>
+      <c r="Z63" s="150"/>
+      <c r="AA63" s="150"/>
+      <c r="AB63" s="150"/>
+      <c r="AC63" s="150"/>
+      <c r="AD63" s="150"/>
+      <c r="AE63" s="150"/>
+      <c r="AF63" s="150"/>
+      <c r="AG63" s="150"/>
+      <c r="AH63" s="150"/>
       <c r="AK63" s="37"/>
       <c r="AO63" s="37"/>
       <c r="AP63" s="37"/>
@@ -7956,42 +7956,42 @@
       <c r="AW63" s="37"/>
     </row>
     <row r="64" spans="1:53" s="2" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A64" s="114" t="s">
+      <c r="A64" s="150" t="s">
         <v>123</v>
       </c>
-      <c r="B64" s="114"/>
-      <c r="C64" s="114"/>
-      <c r="D64" s="114"/>
-      <c r="E64" s="114"/>
-      <c r="F64" s="114"/>
-      <c r="G64" s="114"/>
-      <c r="H64" s="114"/>
-      <c r="I64" s="114"/>
-      <c r="J64" s="114"/>
-      <c r="K64" s="114"/>
-      <c r="L64" s="114"/>
-      <c r="M64" s="114"/>
-      <c r="N64" s="114"/>
-      <c r="O64" s="114"/>
-      <c r="P64" s="114"/>
-      <c r="Q64" s="114"/>
-      <c r="R64" s="114"/>
-      <c r="S64" s="114"/>
-      <c r="T64" s="114"/>
-      <c r="U64" s="114"/>
-      <c r="V64" s="114"/>
-      <c r="W64" s="114"/>
-      <c r="X64" s="114"/>
-      <c r="Y64" s="114"/>
-      <c r="Z64" s="114"/>
-      <c r="AA64" s="114"/>
-      <c r="AB64" s="114"/>
-      <c r="AC64" s="114"/>
-      <c r="AD64" s="114"/>
-      <c r="AE64" s="114"/>
-      <c r="AF64" s="114"/>
-      <c r="AG64" s="114"/>
-      <c r="AH64" s="114"/>
+      <c r="B64" s="150"/>
+      <c r="C64" s="150"/>
+      <c r="D64" s="150"/>
+      <c r="E64" s="150"/>
+      <c r="F64" s="150"/>
+      <c r="G64" s="150"/>
+      <c r="H64" s="150"/>
+      <c r="I64" s="150"/>
+      <c r="J64" s="150"/>
+      <c r="K64" s="150"/>
+      <c r="L64" s="150"/>
+      <c r="M64" s="150"/>
+      <c r="N64" s="150"/>
+      <c r="O64" s="150"/>
+      <c r="P64" s="150"/>
+      <c r="Q64" s="150"/>
+      <c r="R64" s="150"/>
+      <c r="S64" s="150"/>
+      <c r="T64" s="150"/>
+      <c r="U64" s="150"/>
+      <c r="V64" s="150"/>
+      <c r="W64" s="150"/>
+      <c r="X64" s="150"/>
+      <c r="Y64" s="150"/>
+      <c r="Z64" s="150"/>
+      <c r="AA64" s="150"/>
+      <c r="AB64" s="150"/>
+      <c r="AC64" s="150"/>
+      <c r="AD64" s="150"/>
+      <c r="AE64" s="150"/>
+      <c r="AF64" s="150"/>
+      <c r="AG64" s="150"/>
+      <c r="AH64" s="150"/>
       <c r="AK64" s="37"/>
       <c r="AO64" s="37"/>
       <c r="AP64" s="37"/>
@@ -8001,42 +8001,42 @@
       <c r="AW64" s="37"/>
     </row>
     <row r="65" spans="1:53" s="2" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A65" s="114" t="s">
+      <c r="A65" s="150" t="s">
         <v>124</v>
       </c>
-      <c r="B65" s="114"/>
-      <c r="C65" s="114"/>
-      <c r="D65" s="114"/>
-      <c r="E65" s="114"/>
-      <c r="F65" s="114"/>
-      <c r="G65" s="114"/>
-      <c r="H65" s="114"/>
-      <c r="I65" s="114"/>
-      <c r="J65" s="114"/>
-      <c r="K65" s="114"/>
-      <c r="L65" s="114"/>
-      <c r="M65" s="114"/>
-      <c r="N65" s="114"/>
-      <c r="O65" s="114"/>
-      <c r="P65" s="114"/>
-      <c r="Q65" s="114"/>
-      <c r="R65" s="114"/>
-      <c r="S65" s="114"/>
-      <c r="T65" s="114"/>
-      <c r="U65" s="114"/>
-      <c r="V65" s="114"/>
-      <c r="W65" s="114"/>
-      <c r="X65" s="114"/>
-      <c r="Y65" s="114"/>
-      <c r="Z65" s="114"/>
-      <c r="AA65" s="114"/>
-      <c r="AB65" s="114"/>
-      <c r="AC65" s="114"/>
-      <c r="AD65" s="114"/>
-      <c r="AE65" s="114"/>
-      <c r="AF65" s="114"/>
-      <c r="AG65" s="114"/>
-      <c r="AH65" s="114"/>
+      <c r="B65" s="150"/>
+      <c r="C65" s="150"/>
+      <c r="D65" s="150"/>
+      <c r="E65" s="150"/>
+      <c r="F65" s="150"/>
+      <c r="G65" s="150"/>
+      <c r="H65" s="150"/>
+      <c r="I65" s="150"/>
+      <c r="J65" s="150"/>
+      <c r="K65" s="150"/>
+      <c r="L65" s="150"/>
+      <c r="M65" s="150"/>
+      <c r="N65" s="150"/>
+      <c r="O65" s="150"/>
+      <c r="P65" s="150"/>
+      <c r="Q65" s="150"/>
+      <c r="R65" s="150"/>
+      <c r="S65" s="150"/>
+      <c r="T65" s="150"/>
+      <c r="U65" s="150"/>
+      <c r="V65" s="150"/>
+      <c r="W65" s="150"/>
+      <c r="X65" s="150"/>
+      <c r="Y65" s="150"/>
+      <c r="Z65" s="150"/>
+      <c r="AA65" s="150"/>
+      <c r="AB65" s="150"/>
+      <c r="AC65" s="150"/>
+      <c r="AD65" s="150"/>
+      <c r="AE65" s="150"/>
+      <c r="AF65" s="150"/>
+      <c r="AG65" s="150"/>
+      <c r="AH65" s="150"/>
       <c r="AK65" s="37"/>
       <c r="AO65" s="37"/>
       <c r="AP65" s="37"/>
@@ -8046,42 +8046,42 @@
       <c r="AW65" s="37"/>
     </row>
     <row r="66" spans="1:53" s="2" customFormat="1" ht="29" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A66" s="114" t="s">
+      <c r="A66" s="150" t="s">
         <v>125</v>
       </c>
-      <c r="B66" s="114"/>
-      <c r="C66" s="114"/>
-      <c r="D66" s="114"/>
-      <c r="E66" s="114"/>
-      <c r="F66" s="114"/>
-      <c r="G66" s="114"/>
-      <c r="H66" s="114"/>
-      <c r="I66" s="114"/>
-      <c r="J66" s="114"/>
-      <c r="K66" s="114"/>
-      <c r="L66" s="114"/>
-      <c r="M66" s="114"/>
-      <c r="N66" s="114"/>
-      <c r="O66" s="114"/>
-      <c r="P66" s="114"/>
-      <c r="Q66" s="114"/>
-      <c r="R66" s="114"/>
-      <c r="S66" s="114"/>
-      <c r="T66" s="114"/>
-      <c r="U66" s="114"/>
-      <c r="V66" s="114"/>
-      <c r="W66" s="114"/>
-      <c r="X66" s="114"/>
-      <c r="Y66" s="114"/>
-      <c r="Z66" s="114"/>
-      <c r="AA66" s="114"/>
-      <c r="AB66" s="114"/>
-      <c r="AC66" s="114"/>
-      <c r="AD66" s="114"/>
-      <c r="AE66" s="114"/>
-      <c r="AF66" s="114"/>
-      <c r="AG66" s="114"/>
-      <c r="AH66" s="114"/>
+      <c r="B66" s="150"/>
+      <c r="C66" s="150"/>
+      <c r="D66" s="150"/>
+      <c r="E66" s="150"/>
+      <c r="F66" s="150"/>
+      <c r="G66" s="150"/>
+      <c r="H66" s="150"/>
+      <c r="I66" s="150"/>
+      <c r="J66" s="150"/>
+      <c r="K66" s="150"/>
+      <c r="L66" s="150"/>
+      <c r="M66" s="150"/>
+      <c r="N66" s="150"/>
+      <c r="O66" s="150"/>
+      <c r="P66" s="150"/>
+      <c r="Q66" s="150"/>
+      <c r="R66" s="150"/>
+      <c r="S66" s="150"/>
+      <c r="T66" s="150"/>
+      <c r="U66" s="150"/>
+      <c r="V66" s="150"/>
+      <c r="W66" s="150"/>
+      <c r="X66" s="150"/>
+      <c r="Y66" s="150"/>
+      <c r="Z66" s="150"/>
+      <c r="AA66" s="150"/>
+      <c r="AB66" s="150"/>
+      <c r="AC66" s="150"/>
+      <c r="AD66" s="150"/>
+      <c r="AE66" s="150"/>
+      <c r="AF66" s="150"/>
+      <c r="AG66" s="150"/>
+      <c r="AH66" s="150"/>
       <c r="AI66" s="22"/>
       <c r="AJ66" s="22"/>
       <c r="AK66" s="37"/>
@@ -8093,42 +8093,42 @@
       <c r="AW66" s="37"/>
     </row>
     <row r="67" spans="1:53" s="22" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A67" s="114" t="s">
+      <c r="A67" s="150" t="s">
         <v>126</v>
       </c>
-      <c r="B67" s="114"/>
-      <c r="C67" s="114"/>
-      <c r="D67" s="114"/>
-      <c r="E67" s="114"/>
-      <c r="F67" s="114"/>
-      <c r="G67" s="114"/>
-      <c r="H67" s="114"/>
-      <c r="I67" s="114"/>
-      <c r="J67" s="114"/>
-      <c r="K67" s="114"/>
-      <c r="L67" s="114"/>
-      <c r="M67" s="114"/>
-      <c r="N67" s="114"/>
-      <c r="O67" s="114"/>
-      <c r="P67" s="114"/>
-      <c r="Q67" s="114"/>
-      <c r="R67" s="114"/>
-      <c r="S67" s="114"/>
-      <c r="T67" s="114"/>
-      <c r="U67" s="114"/>
-      <c r="V67" s="114"/>
-      <c r="W67" s="114"/>
-      <c r="X67" s="114"/>
-      <c r="Y67" s="114"/>
-      <c r="Z67" s="114"/>
-      <c r="AA67" s="114"/>
-      <c r="AB67" s="114"/>
-      <c r="AC67" s="114"/>
-      <c r="AD67" s="114"/>
-      <c r="AE67" s="114"/>
-      <c r="AF67" s="114"/>
-      <c r="AG67" s="114"/>
-      <c r="AH67" s="114"/>
+      <c r="B67" s="150"/>
+      <c r="C67" s="150"/>
+      <c r="D67" s="150"/>
+      <c r="E67" s="150"/>
+      <c r="F67" s="150"/>
+      <c r="G67" s="150"/>
+      <c r="H67" s="150"/>
+      <c r="I67" s="150"/>
+      <c r="J67" s="150"/>
+      <c r="K67" s="150"/>
+      <c r="L67" s="150"/>
+      <c r="M67" s="150"/>
+      <c r="N67" s="150"/>
+      <c r="O67" s="150"/>
+      <c r="P67" s="150"/>
+      <c r="Q67" s="150"/>
+      <c r="R67" s="150"/>
+      <c r="S67" s="150"/>
+      <c r="T67" s="150"/>
+      <c r="U67" s="150"/>
+      <c r="V67" s="150"/>
+      <c r="W67" s="150"/>
+      <c r="X67" s="150"/>
+      <c r="Y67" s="150"/>
+      <c r="Z67" s="150"/>
+      <c r="AA67" s="150"/>
+      <c r="AB67" s="150"/>
+      <c r="AC67" s="150"/>
+      <c r="AD67" s="150"/>
+      <c r="AE67" s="150"/>
+      <c r="AF67" s="150"/>
+      <c r="AG67" s="150"/>
+      <c r="AH67" s="150"/>
       <c r="AI67" s="2"/>
       <c r="AJ67" s="2"/>
       <c r="AK67" s="37"/>
@@ -8150,42 +8150,42 @@
       <c r="BA67" s="2"/>
     </row>
     <row r="68" spans="1:53" s="2" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A68" s="114" t="s">
+      <c r="A68" s="150" t="s">
         <v>127</v>
       </c>
-      <c r="B68" s="114"/>
-      <c r="C68" s="114"/>
-      <c r="D68" s="114"/>
-      <c r="E68" s="114"/>
-      <c r="F68" s="114"/>
-      <c r="G68" s="114"/>
-      <c r="H68" s="114"/>
-      <c r="I68" s="114"/>
-      <c r="J68" s="114"/>
-      <c r="K68" s="114"/>
-      <c r="L68" s="114"/>
-      <c r="M68" s="114"/>
-      <c r="N68" s="114"/>
-      <c r="O68" s="114"/>
-      <c r="P68" s="114"/>
-      <c r="Q68" s="114"/>
-      <c r="R68" s="114"/>
-      <c r="S68" s="114"/>
-      <c r="T68" s="114"/>
-      <c r="U68" s="114"/>
-      <c r="V68" s="114"/>
-      <c r="W68" s="114"/>
-      <c r="X68" s="114"/>
-      <c r="Y68" s="114"/>
-      <c r="Z68" s="114"/>
-      <c r="AA68" s="114"/>
-      <c r="AB68" s="114"/>
-      <c r="AC68" s="114"/>
-      <c r="AD68" s="114"/>
-      <c r="AE68" s="114"/>
-      <c r="AF68" s="114"/>
-      <c r="AG68" s="114"/>
-      <c r="AH68" s="114"/>
+      <c r="B68" s="150"/>
+      <c r="C68" s="150"/>
+      <c r="D68" s="150"/>
+      <c r="E68" s="150"/>
+      <c r="F68" s="150"/>
+      <c r="G68" s="150"/>
+      <c r="H68" s="150"/>
+      <c r="I68" s="150"/>
+      <c r="J68" s="150"/>
+      <c r="K68" s="150"/>
+      <c r="L68" s="150"/>
+      <c r="M68" s="150"/>
+      <c r="N68" s="150"/>
+      <c r="O68" s="150"/>
+      <c r="P68" s="150"/>
+      <c r="Q68" s="150"/>
+      <c r="R68" s="150"/>
+      <c r="S68" s="150"/>
+      <c r="T68" s="150"/>
+      <c r="U68" s="150"/>
+      <c r="V68" s="150"/>
+      <c r="W68" s="150"/>
+      <c r="X68" s="150"/>
+      <c r="Y68" s="150"/>
+      <c r="Z68" s="150"/>
+      <c r="AA68" s="150"/>
+      <c r="AB68" s="150"/>
+      <c r="AC68" s="150"/>
+      <c r="AD68" s="150"/>
+      <c r="AE68" s="150"/>
+      <c r="AF68" s="150"/>
+      <c r="AG68" s="150"/>
+      <c r="AH68" s="150"/>
       <c r="AK68" s="42"/>
       <c r="AN68" s="22"/>
       <c r="AO68" s="37"/>
@@ -8196,42 +8196,42 @@
       <c r="AW68" s="37"/>
     </row>
     <row r="69" spans="1:53" s="2" customFormat="1" ht="23" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A69" s="114" t="s">
+      <c r="A69" s="150" t="s">
         <v>128</v>
       </c>
-      <c r="B69" s="114"/>
-      <c r="C69" s="114"/>
-      <c r="D69" s="114"/>
-      <c r="E69" s="114"/>
-      <c r="F69" s="114"/>
-      <c r="G69" s="114"/>
-      <c r="H69" s="114"/>
-      <c r="I69" s="114"/>
-      <c r="J69" s="114"/>
-      <c r="K69" s="114"/>
-      <c r="L69" s="114"/>
-      <c r="M69" s="114"/>
-      <c r="N69" s="114"/>
-      <c r="O69" s="114"/>
-      <c r="P69" s="114"/>
-      <c r="Q69" s="114"/>
-      <c r="R69" s="114"/>
-      <c r="S69" s="114"/>
-      <c r="T69" s="114"/>
-      <c r="U69" s="114"/>
-      <c r="V69" s="114"/>
-      <c r="W69" s="114"/>
-      <c r="X69" s="114"/>
-      <c r="Y69" s="114"/>
-      <c r="Z69" s="114"/>
-      <c r="AA69" s="114"/>
-      <c r="AB69" s="114"/>
-      <c r="AC69" s="114"/>
-      <c r="AD69" s="114"/>
-      <c r="AE69" s="114"/>
-      <c r="AF69" s="114"/>
-      <c r="AG69" s="114"/>
-      <c r="AH69" s="114"/>
+      <c r="B69" s="150"/>
+      <c r="C69" s="150"/>
+      <c r="D69" s="150"/>
+      <c r="E69" s="150"/>
+      <c r="F69" s="150"/>
+      <c r="G69" s="150"/>
+      <c r="H69" s="150"/>
+      <c r="I69" s="150"/>
+      <c r="J69" s="150"/>
+      <c r="K69" s="150"/>
+      <c r="L69" s="150"/>
+      <c r="M69" s="150"/>
+      <c r="N69" s="150"/>
+      <c r="O69" s="150"/>
+      <c r="P69" s="150"/>
+      <c r="Q69" s="150"/>
+      <c r="R69" s="150"/>
+      <c r="S69" s="150"/>
+      <c r="T69" s="150"/>
+      <c r="U69" s="150"/>
+      <c r="V69" s="150"/>
+      <c r="W69" s="150"/>
+      <c r="X69" s="150"/>
+      <c r="Y69" s="150"/>
+      <c r="Z69" s="150"/>
+      <c r="AA69" s="150"/>
+      <c r="AB69" s="150"/>
+      <c r="AC69" s="150"/>
+      <c r="AD69" s="150"/>
+      <c r="AE69" s="150"/>
+      <c r="AF69" s="150"/>
+      <c r="AG69" s="150"/>
+      <c r="AH69" s="150"/>
       <c r="AK69" s="37"/>
       <c r="AL69" s="22"/>
       <c r="AM69" s="22"/>
@@ -8245,42 +8245,42 @@
       <c r="AZ69" s="22"/>
     </row>
     <row r="70" spans="1:53" s="2" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A70" s="114" t="s">
+      <c r="A70" s="150" t="s">
         <v>129</v>
       </c>
-      <c r="B70" s="114"/>
-      <c r="C70" s="114"/>
-      <c r="D70" s="114"/>
-      <c r="E70" s="114"/>
-      <c r="F70" s="114"/>
-      <c r="G70" s="114"/>
-      <c r="H70" s="114"/>
-      <c r="I70" s="114"/>
-      <c r="J70" s="114"/>
-      <c r="K70" s="114"/>
-      <c r="L70" s="114"/>
-      <c r="M70" s="114"/>
-      <c r="N70" s="114"/>
-      <c r="O70" s="114"/>
-      <c r="P70" s="114"/>
-      <c r="Q70" s="114"/>
-      <c r="R70" s="114"/>
-      <c r="S70" s="114"/>
-      <c r="T70" s="114"/>
-      <c r="U70" s="114"/>
-      <c r="V70" s="114"/>
-      <c r="W70" s="114"/>
-      <c r="X70" s="114"/>
-      <c r="Y70" s="114"/>
-      <c r="Z70" s="114"/>
-      <c r="AA70" s="114"/>
-      <c r="AB70" s="114"/>
-      <c r="AC70" s="114"/>
-      <c r="AD70" s="114"/>
-      <c r="AE70" s="114"/>
-      <c r="AF70" s="114"/>
-      <c r="AG70" s="114"/>
-      <c r="AH70" s="114"/>
+      <c r="B70" s="150"/>
+      <c r="C70" s="150"/>
+      <c r="D70" s="150"/>
+      <c r="E70" s="150"/>
+      <c r="F70" s="150"/>
+      <c r="G70" s="150"/>
+      <c r="H70" s="150"/>
+      <c r="I70" s="150"/>
+      <c r="J70" s="150"/>
+      <c r="K70" s="150"/>
+      <c r="L70" s="150"/>
+      <c r="M70" s="150"/>
+      <c r="N70" s="150"/>
+      <c r="O70" s="150"/>
+      <c r="P70" s="150"/>
+      <c r="Q70" s="150"/>
+      <c r="R70" s="150"/>
+      <c r="S70" s="150"/>
+      <c r="T70" s="150"/>
+      <c r="U70" s="150"/>
+      <c r="V70" s="150"/>
+      <c r="W70" s="150"/>
+      <c r="X70" s="150"/>
+      <c r="Y70" s="150"/>
+      <c r="Z70" s="150"/>
+      <c r="AA70" s="150"/>
+      <c r="AB70" s="150"/>
+      <c r="AC70" s="150"/>
+      <c r="AD70" s="150"/>
+      <c r="AE70" s="150"/>
+      <c r="AF70" s="150"/>
+      <c r="AG70" s="150"/>
+      <c r="AH70" s="150"/>
       <c r="AK70" s="37"/>
       <c r="AO70" s="37"/>
       <c r="AP70" s="37"/>
@@ -8295,42 +8295,42 @@
       <c r="BA70" s="22"/>
     </row>
     <row r="71" spans="1:53" s="2" customFormat="1" ht="29.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A71" s="114" t="s">
+      <c r="A71" s="150" t="s">
         <v>130</v>
       </c>
-      <c r="B71" s="114"/>
-      <c r="C71" s="114"/>
-      <c r="D71" s="114"/>
-      <c r="E71" s="114"/>
-      <c r="F71" s="114"/>
-      <c r="G71" s="114"/>
-      <c r="H71" s="114"/>
-      <c r="I71" s="114"/>
-      <c r="J71" s="114"/>
-      <c r="K71" s="114"/>
-      <c r="L71" s="114"/>
-      <c r="M71" s="114"/>
-      <c r="N71" s="114"/>
-      <c r="O71" s="114"/>
-      <c r="P71" s="114"/>
-      <c r="Q71" s="114"/>
-      <c r="R71" s="114"/>
-      <c r="S71" s="114"/>
-      <c r="T71" s="114"/>
-      <c r="U71" s="114"/>
-      <c r="V71" s="114"/>
-      <c r="W71" s="114"/>
-      <c r="X71" s="114"/>
-      <c r="Y71" s="114"/>
-      <c r="Z71" s="114"/>
-      <c r="AA71" s="114"/>
-      <c r="AB71" s="114"/>
-      <c r="AC71" s="114"/>
-      <c r="AD71" s="114"/>
-      <c r="AE71" s="114"/>
-      <c r="AF71" s="114"/>
-      <c r="AG71" s="114"/>
-      <c r="AH71" s="114"/>
+      <c r="B71" s="150"/>
+      <c r="C71" s="150"/>
+      <c r="D71" s="150"/>
+      <c r="E71" s="150"/>
+      <c r="F71" s="150"/>
+      <c r="G71" s="150"/>
+      <c r="H71" s="150"/>
+      <c r="I71" s="150"/>
+      <c r="J71" s="150"/>
+      <c r="K71" s="150"/>
+      <c r="L71" s="150"/>
+      <c r="M71" s="150"/>
+      <c r="N71" s="150"/>
+      <c r="O71" s="150"/>
+      <c r="P71" s="150"/>
+      <c r="Q71" s="150"/>
+      <c r="R71" s="150"/>
+      <c r="S71" s="150"/>
+      <c r="T71" s="150"/>
+      <c r="U71" s="150"/>
+      <c r="V71" s="150"/>
+      <c r="W71" s="150"/>
+      <c r="X71" s="150"/>
+      <c r="Y71" s="150"/>
+      <c r="Z71" s="150"/>
+      <c r="AA71" s="150"/>
+      <c r="AB71" s="150"/>
+      <c r="AC71" s="150"/>
+      <c r="AD71" s="150"/>
+      <c r="AE71" s="150"/>
+      <c r="AF71" s="150"/>
+      <c r="AG71" s="150"/>
+      <c r="AH71" s="150"/>
       <c r="AK71" s="37"/>
       <c r="AO71" s="37"/>
       <c r="AP71" s="37"/>
@@ -8490,6 +8490,119 @@
     </customSheetView>
   </customSheetViews>
   <mergeCells count="137">
+    <mergeCell ref="AW10:AX10"/>
+    <mergeCell ref="AU30:AY31"/>
+    <mergeCell ref="AK8:AK9"/>
+    <mergeCell ref="AL8:AL9"/>
+    <mergeCell ref="AZ30:AZ31"/>
+    <mergeCell ref="A20:A21"/>
+    <mergeCell ref="AF16:AF17"/>
+    <mergeCell ref="AG16:AG17"/>
+    <mergeCell ref="A18:A19"/>
+    <mergeCell ref="AG14:AG15"/>
+    <mergeCell ref="A16:A17"/>
+    <mergeCell ref="A14:A15"/>
+    <mergeCell ref="AW11:AX11"/>
+    <mergeCell ref="AD3:AG3"/>
+    <mergeCell ref="A3:H3"/>
+    <mergeCell ref="A4:H4"/>
+    <mergeCell ref="M6:T6"/>
+    <mergeCell ref="B6:I6"/>
+    <mergeCell ref="U6:AC6"/>
+    <mergeCell ref="AD6:AH6"/>
+    <mergeCell ref="AE12:AE13"/>
+    <mergeCell ref="AF12:AF13"/>
+    <mergeCell ref="AG12:AG13"/>
+    <mergeCell ref="AG10:AG11"/>
+    <mergeCell ref="A12:A13"/>
+    <mergeCell ref="Y3:AC3"/>
+    <mergeCell ref="A7:A9"/>
+    <mergeCell ref="B8:AF8"/>
+    <mergeCell ref="B7:AF7"/>
+    <mergeCell ref="A10:A11"/>
+    <mergeCell ref="Y4:AC4"/>
+    <mergeCell ref="AD4:AH4"/>
+    <mergeCell ref="AG34:AG35"/>
+    <mergeCell ref="O34:AF35"/>
+    <mergeCell ref="A1:AH2"/>
+    <mergeCell ref="I3:X3"/>
+    <mergeCell ref="I4:X4"/>
+    <mergeCell ref="J6:L6"/>
+    <mergeCell ref="A5:AH5"/>
+    <mergeCell ref="AG32:AG33"/>
+    <mergeCell ref="AG30:AG31"/>
+    <mergeCell ref="A32:A33"/>
+    <mergeCell ref="AF30:AF31"/>
+    <mergeCell ref="A30:A31"/>
+    <mergeCell ref="AG28:AG29"/>
+    <mergeCell ref="AG26:AG27"/>
+    <mergeCell ref="A28:A29"/>
+    <mergeCell ref="AF26:AF27"/>
+    <mergeCell ref="AG24:AG25"/>
+    <mergeCell ref="A26:A27"/>
+    <mergeCell ref="AG22:AG23"/>
+    <mergeCell ref="A24:A25"/>
+    <mergeCell ref="A22:A23"/>
+    <mergeCell ref="AF20:AF21"/>
+    <mergeCell ref="AG20:AG21"/>
+    <mergeCell ref="AG18:AG19"/>
+    <mergeCell ref="A70:AH70"/>
+    <mergeCell ref="A71:AH71"/>
+    <mergeCell ref="A37:AF37"/>
+    <mergeCell ref="AD38:AF38"/>
+    <mergeCell ref="AA38:AC38"/>
+    <mergeCell ref="AD39:AF39"/>
+    <mergeCell ref="A64:AH64"/>
+    <mergeCell ref="A65:AH65"/>
+    <mergeCell ref="A66:AH66"/>
+    <mergeCell ref="A67:AH67"/>
+    <mergeCell ref="A68:AH68"/>
+    <mergeCell ref="A69:AH69"/>
+    <mergeCell ref="A61:AH61"/>
+    <mergeCell ref="A60:AH60"/>
+    <mergeCell ref="A62:AH62"/>
+    <mergeCell ref="A63:AH63"/>
+    <mergeCell ref="AD40:AF40"/>
+    <mergeCell ref="AD41:AF41"/>
+    <mergeCell ref="AD42:AF42"/>
+    <mergeCell ref="AD43:AF43"/>
+    <mergeCell ref="R40:T40"/>
+    <mergeCell ref="U40:W40"/>
+    <mergeCell ref="X40:Z40"/>
+    <mergeCell ref="O41:Q41"/>
+    <mergeCell ref="AD44:AF44"/>
+    <mergeCell ref="AD45:AF45"/>
+    <mergeCell ref="AA39:AC39"/>
+    <mergeCell ref="AA40:AC40"/>
+    <mergeCell ref="AA41:AC41"/>
+    <mergeCell ref="AA42:AC42"/>
+    <mergeCell ref="AA43:AC43"/>
+    <mergeCell ref="AA44:AC44"/>
+    <mergeCell ref="AA45:AC45"/>
+    <mergeCell ref="Z58:AH58"/>
+    <mergeCell ref="Z56:AH57"/>
+    <mergeCell ref="A58:K58"/>
+    <mergeCell ref="T56:Y57"/>
+    <mergeCell ref="N38:Z38"/>
+    <mergeCell ref="A38:D38"/>
+    <mergeCell ref="E38:G38"/>
+    <mergeCell ref="H38:M38"/>
+    <mergeCell ref="A52:T52"/>
+    <mergeCell ref="A53:N53"/>
+    <mergeCell ref="O53:Q53"/>
+    <mergeCell ref="R53:T53"/>
+    <mergeCell ref="A45:W45"/>
+    <mergeCell ref="X45:Z45"/>
+    <mergeCell ref="O49:Q49"/>
+    <mergeCell ref="R49:T49"/>
+    <mergeCell ref="A48:N48"/>
+    <mergeCell ref="A47:T47"/>
+    <mergeCell ref="B50:N50"/>
+    <mergeCell ref="O50:T50"/>
+    <mergeCell ref="O48:Q48"/>
+    <mergeCell ref="R48:T48"/>
+    <mergeCell ref="B49:N49"/>
+    <mergeCell ref="O43:Q43"/>
     <mergeCell ref="O54:Q54"/>
     <mergeCell ref="R54:T54"/>
     <mergeCell ref="A54:N54"/>
@@ -8514,119 +8627,6 @@
     <mergeCell ref="B44:Z44"/>
     <mergeCell ref="O39:Q39"/>
     <mergeCell ref="O40:Q40"/>
-    <mergeCell ref="Z58:AH58"/>
-    <mergeCell ref="Z56:AH57"/>
-    <mergeCell ref="A58:K58"/>
-    <mergeCell ref="T56:Y57"/>
-    <mergeCell ref="N38:Z38"/>
-    <mergeCell ref="A38:D38"/>
-    <mergeCell ref="E38:G38"/>
-    <mergeCell ref="H38:M38"/>
-    <mergeCell ref="A52:T52"/>
-    <mergeCell ref="A53:N53"/>
-    <mergeCell ref="O53:Q53"/>
-    <mergeCell ref="R53:T53"/>
-    <mergeCell ref="A45:W45"/>
-    <mergeCell ref="X45:Z45"/>
-    <mergeCell ref="O49:Q49"/>
-    <mergeCell ref="R49:T49"/>
-    <mergeCell ref="A48:N48"/>
-    <mergeCell ref="A47:T47"/>
-    <mergeCell ref="B50:N50"/>
-    <mergeCell ref="O50:T50"/>
-    <mergeCell ref="O48:Q48"/>
-    <mergeCell ref="R48:T48"/>
-    <mergeCell ref="B49:N49"/>
-    <mergeCell ref="O43:Q43"/>
-    <mergeCell ref="AD44:AF44"/>
-    <mergeCell ref="AD45:AF45"/>
-    <mergeCell ref="AA39:AC39"/>
-    <mergeCell ref="AA40:AC40"/>
-    <mergeCell ref="AA41:AC41"/>
-    <mergeCell ref="AA42:AC42"/>
-    <mergeCell ref="AA43:AC43"/>
-    <mergeCell ref="AA44:AC44"/>
-    <mergeCell ref="AA45:AC45"/>
-    <mergeCell ref="A70:AH70"/>
-    <mergeCell ref="A71:AH71"/>
-    <mergeCell ref="A37:AF37"/>
-    <mergeCell ref="AD38:AF38"/>
-    <mergeCell ref="AA38:AC38"/>
-    <mergeCell ref="AD39:AF39"/>
-    <mergeCell ref="A64:AH64"/>
-    <mergeCell ref="A65:AH65"/>
-    <mergeCell ref="A66:AH66"/>
-    <mergeCell ref="A67:AH67"/>
-    <mergeCell ref="A68:AH68"/>
-    <mergeCell ref="A69:AH69"/>
-    <mergeCell ref="A61:AH61"/>
-    <mergeCell ref="A60:AH60"/>
-    <mergeCell ref="A62:AH62"/>
-    <mergeCell ref="A63:AH63"/>
-    <mergeCell ref="AD40:AF40"/>
-    <mergeCell ref="AD41:AF41"/>
-    <mergeCell ref="AD42:AF42"/>
-    <mergeCell ref="AD43:AF43"/>
-    <mergeCell ref="R40:T40"/>
-    <mergeCell ref="U40:W40"/>
-    <mergeCell ref="X40:Z40"/>
-    <mergeCell ref="O41:Q41"/>
-    <mergeCell ref="AG34:AG35"/>
-    <mergeCell ref="O34:AF35"/>
-    <mergeCell ref="A1:AH2"/>
-    <mergeCell ref="I3:X3"/>
-    <mergeCell ref="I4:X4"/>
-    <mergeCell ref="J6:L6"/>
-    <mergeCell ref="A5:AH5"/>
-    <mergeCell ref="AG32:AG33"/>
-    <mergeCell ref="AG30:AG31"/>
-    <mergeCell ref="A32:A33"/>
-    <mergeCell ref="AF30:AF31"/>
-    <mergeCell ref="A30:A31"/>
-    <mergeCell ref="AG28:AG29"/>
-    <mergeCell ref="AG26:AG27"/>
-    <mergeCell ref="A28:A29"/>
-    <mergeCell ref="AF26:AF27"/>
-    <mergeCell ref="AG24:AG25"/>
-    <mergeCell ref="A26:A27"/>
-    <mergeCell ref="AG22:AG23"/>
-    <mergeCell ref="A24:A25"/>
-    <mergeCell ref="A22:A23"/>
-    <mergeCell ref="AF20:AF21"/>
-    <mergeCell ref="AG20:AG21"/>
-    <mergeCell ref="AG18:AG19"/>
-    <mergeCell ref="AD3:AG3"/>
-    <mergeCell ref="A3:H3"/>
-    <mergeCell ref="A4:H4"/>
-    <mergeCell ref="M6:T6"/>
-    <mergeCell ref="B6:I6"/>
-    <mergeCell ref="U6:AC6"/>
-    <mergeCell ref="AD6:AH6"/>
-    <mergeCell ref="AE12:AE13"/>
-    <mergeCell ref="AF12:AF13"/>
-    <mergeCell ref="AG12:AG13"/>
-    <mergeCell ref="AG10:AG11"/>
-    <mergeCell ref="A12:A13"/>
-    <mergeCell ref="Y3:AC3"/>
-    <mergeCell ref="A7:A9"/>
-    <mergeCell ref="B8:AF8"/>
-    <mergeCell ref="B7:AF7"/>
-    <mergeCell ref="A10:A11"/>
-    <mergeCell ref="Y4:AC4"/>
-    <mergeCell ref="AD4:AH4"/>
-    <mergeCell ref="AW10:AX10"/>
-    <mergeCell ref="AU30:AY31"/>
-    <mergeCell ref="AK8:AK9"/>
-    <mergeCell ref="AL8:AL9"/>
-    <mergeCell ref="AZ30:AZ31"/>
-    <mergeCell ref="A20:A21"/>
-    <mergeCell ref="AF16:AF17"/>
-    <mergeCell ref="AG16:AG17"/>
-    <mergeCell ref="A18:A19"/>
-    <mergeCell ref="AG14:AG15"/>
-    <mergeCell ref="A16:A17"/>
-    <mergeCell ref="A14:A15"/>
-    <mergeCell ref="AW11:AX11"/>
   </mergeCells>
   <conditionalFormatting sqref="B12:AD12">
     <cfRule type="expression" dxfId="48" priority="95">
@@ -8847,6 +8847,27 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <Pojekttitel xmlns="aaf634d5-3b14-4b2e-9e8a-d5e4de058a1f" xsi:nil="true"/>
+    <TaxCatchAll xmlns="d773664d-3496-4791-87fd-7864084b790e" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="aaf634d5-3b14-4b2e-9e8a-d5e4de058a1f">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Dokument" ma:contentTypeID="0x0101008C3277064969C648B4B388B3EF6677A1" ma:contentTypeVersion="21" ma:contentTypeDescription="Ein neues Dokument erstellen." ma:contentTypeScope="" ma:versionID="755dff11402872183bc692b327197892">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="aaf634d5-3b14-4b2e-9e8a-d5e4de058a1f" xmlns:ns3="d773664d-3496-4791-87fd-7864084b790e" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="a9faaf0febccef147102967eb6808013" ns2:_="" ns3:_="">
     <xsd:import namespace="aaf634d5-3b14-4b2e-9e8a-d5e4de058a1f"/>
@@ -9109,28 +9130,32 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{68ACEC69-B141-4E17-BC68-1F734A38FB8A}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="aaf634d5-3b14-4b2e-9e8a-d5e4de058a1f"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="d773664d-3496-4791-87fd-7864084b790e"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <Pojekttitel xmlns="aaf634d5-3b14-4b2e-9e8a-d5e4de058a1f" xsi:nil="true"/>
-    <TaxCatchAll xmlns="d773664d-3496-4791-87fd-7864084b790e" xsi:nil="true"/>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="aaf634d5-3b14-4b2e-9e8a-d5e4de058a1f">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-  </documentManagement>
-</p:properties>
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{9BB6DB75-B68B-46AA-9AE1-8A34269744CC}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{02C7C122-7BD2-4019-B750-C18FE818D264}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -9147,29 +9172,4 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{9BB6DB75-B68B-46AA-9AE1-8A34269744CC}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{68ACEC69-B141-4E17-BC68-1F734A38FB8A}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="aaf634d5-3b14-4b2e-9e8a-d5e4de058a1f"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="d773664d-3496-4791-87fd-7864084b790e"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
 </file>
</xml_diff>